<commit_message>
Mogut MovimentCompra de Producte a Moviment. Afegit Test
--HG--
branch : Troba preu orig. fons
</commit_message>
<xml_diff>
--- a/Docs/CompresOriginals.xlsx
+++ b/Docs/CompresOriginals.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4507"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="80" yWindow="130" windowWidth="19140" windowHeight="7830" activeTab="2"/>
+    <workbookView xWindow="80" yWindow="130" windowWidth="19140" windowHeight="7830" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet5" sheetId="7" r:id="rId1"/>
@@ -12,6 +12,7 @@
     <sheet name="Sheet3" sheetId="5" r:id="rId3"/>
     <sheet name="Sheet2" sheetId="4" r:id="rId4"/>
     <sheet name="Sheet1" sheetId="1" r:id="rId5"/>
+    <sheet name="Taula Moviments Sencera" sheetId="8" r:id="rId6"/>
   </sheets>
   <calcPr calcId="125725"/>
 </workbook>
@@ -56,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="120">
   <si>
     <t>Compra</t>
   </si>
@@ -338,13 +339,91 @@
   </si>
   <si>
     <t>Preu U Ori</t>
+  </si>
+  <si>
+    <t>UsuariId</t>
+  </si>
+  <si>
+    <t>ProdId</t>
+  </si>
+  <si>
+    <t>Participacions</t>
+  </si>
+  <si>
+    <t>Despeses</t>
+  </si>
+  <si>
+    <t>Descripcio</t>
+  </si>
+  <si>
+    <t>Traspàs a: DWS AKTIEN STRAT DEUTSCHLAND.</t>
+  </si>
+  <si>
+    <t>ContraSplit. Factor conversor: 3. Preu operació: 7,6.</t>
+  </si>
+  <si>
+    <t>Ampliació de capital de Santander.</t>
+  </si>
+  <si>
+    <t>He sumat varies despesses anteriors.</t>
+  </si>
+  <si>
+    <t>Acumulades despeses antigues.</t>
+  </si>
+  <si>
+    <t>Acumulo despeses antigues. Son tres accions que no tenen cost.</t>
+  </si>
+  <si>
+    <t>Primera compra a SelfBank.</t>
+  </si>
+  <si>
+    <t>Venda ActivoBank.</t>
+  </si>
+  <si>
+    <t>Ampliació de capital de Telefònica.</t>
+  </si>
+  <si>
+    <t>Import net: 1.491,84 €</t>
+  </si>
+  <si>
+    <t>Traspasat a: Fidelity Funds - Indonesia Fund Y-Acc-USD</t>
+  </si>
+  <si>
+    <t>Venda total</t>
+  </si>
+  <si>
+    <t>Compra inicial</t>
+  </si>
+  <si>
+    <t>ContraSplit. Factor conversor: 3. Preu operació: 7,3.</t>
+  </si>
+  <si>
+    <t>Dividendo en acciones.</t>
+  </si>
+  <si>
+    <t>Interessos lloguer accions.</t>
+  </si>
+  <si>
+    <t>ProdId Traspas</t>
+  </si>
+  <si>
+    <t>MovId Venda</t>
+  </si>
+  <si>
+    <t>Preu Participacio</t>
+  </si>
+  <si>
+    <t>Preu Participacio Origen</t>
+  </si>
+  <si>
+    <t>Part acum</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="10">
     <numFmt numFmtId="8" formatCode="#,##0.00\ &quot;€&quot;;[Red]\-#,##0.00\ &quot;€&quot;"/>
     <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
     <numFmt numFmtId="165" formatCode="#,##0.000"/>
@@ -352,6 +431,9 @@
     <numFmt numFmtId="167" formatCode="#,##0.000\ &quot;€&quot;"/>
     <numFmt numFmtId="168" formatCode="0.0000"/>
     <numFmt numFmtId="169" formatCode="#,##0.0000\ &quot;€&quot;"/>
+    <numFmt numFmtId="170" formatCode="#,##0.000\ &quot;€&quot;;[Red]\-#,##0.000\ &quot;€&quot;"/>
+    <numFmt numFmtId="171" formatCode="#,##0.0000\ &quot;€&quot;;[Red]\-#,##0.0000\ &quot;€&quot;"/>
+    <numFmt numFmtId="172" formatCode="#,##0.000_ ;[Red]\-#,##0.000\ "/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -487,7 +569,7 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -562,6 +644,22 @@
     <xf numFmtId="164" fontId="2" fillId="3" borderId="0" xfId="2" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="0" xfId="1" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="170" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="171" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="172" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Bad" xfId="5" builtinId="27"/>
@@ -5894,4 +5992,4737 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:N145"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="8.54296875" style="59" customWidth="1"/>
+    <col min="2" max="2" width="7.90625" style="59" customWidth="1"/>
+    <col min="3" max="3" width="5.7265625" style="59" customWidth="1"/>
+    <col min="4" max="4" width="0" style="59" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="8.7265625" style="59"/>
+    <col min="6" max="7" width="10.08984375" style="75" customWidth="1"/>
+    <col min="8" max="9" width="8.7265625" style="59"/>
+    <col min="10" max="10" width="16.1796875" style="59" customWidth="1"/>
+    <col min="11" max="12" width="11.26953125" style="73" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.7265625" style="71"/>
+    <col min="14" max="14" width="47" style="59" customWidth="1"/>
+    <col min="15" max="16384" width="8.7265625" style="59"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" ht="43.5">
+      <c r="A1" s="69" t="s">
+        <v>94</v>
+      </c>
+      <c r="B1" s="69" t="s">
+        <v>95</v>
+      </c>
+      <c r="C1" s="69" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="69" t="s">
+        <v>59</v>
+      </c>
+      <c r="E1" s="69" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1" s="74" t="s">
+        <v>96</v>
+      </c>
+      <c r="G1" s="74" t="s">
+        <v>119</v>
+      </c>
+      <c r="H1" s="69" t="s">
+        <v>115</v>
+      </c>
+      <c r="I1" s="69" t="s">
+        <v>116</v>
+      </c>
+      <c r="J1" s="69" t="s">
+        <v>62</v>
+      </c>
+      <c r="K1" s="72" t="s">
+        <v>118</v>
+      </c>
+      <c r="L1" s="72" t="s">
+        <v>117</v>
+      </c>
+      <c r="M1" s="70" t="s">
+        <v>97</v>
+      </c>
+      <c r="N1" s="69" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
+      <c r="A2" s="59">
+        <v>1</v>
+      </c>
+      <c r="B2" s="59">
+        <v>1</v>
+      </c>
+      <c r="C2" s="59">
+        <v>27</v>
+      </c>
+      <c r="D2" s="59">
+        <v>0</v>
+      </c>
+      <c r="E2" s="59" t="str">
+        <f>IF(D2=0,"Compra","Venda")</f>
+        <v>Compra</v>
+      </c>
+      <c r="F2" s="75">
+        <v>58.502000000000002</v>
+      </c>
+      <c r="G2" s="75">
+        <f>F2</f>
+        <v>58.502000000000002</v>
+      </c>
+      <c r="J2" s="68">
+        <v>41521</v>
+      </c>
+      <c r="K2" s="73">
+        <v>17.093299999999999</v>
+      </c>
+      <c r="L2" s="73">
+        <v>17.093261768828398</v>
+      </c>
+      <c r="N2" s="59" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3" s="59">
+        <v>1</v>
+      </c>
+      <c r="B3" s="59">
+        <v>1</v>
+      </c>
+      <c r="C3" s="59">
+        <v>29</v>
+      </c>
+      <c r="D3" s="59">
+        <v>0</v>
+      </c>
+      <c r="E3" s="59" t="str">
+        <f>IF(D3=0,"Compra","Venda")</f>
+        <v>Compra</v>
+      </c>
+      <c r="F3" s="75">
+        <v>2347.326</v>
+      </c>
+      <c r="G3" s="75">
+        <f>G2+IF(D3=0,F3,-F3)</f>
+        <v>2405.828</v>
+      </c>
+      <c r="H3" s="59">
+        <v>5</v>
+      </c>
+      <c r="I3" s="59">
+        <v>28</v>
+      </c>
+      <c r="J3" s="68">
+        <v>41794.000011574077</v>
+      </c>
+      <c r="K3" s="73">
+        <v>19.410499999999999</v>
+      </c>
+      <c r="L3" s="73">
+        <v>18.249684960674401</v>
+      </c>
+      <c r="N3" s="59" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
+      <c r="A4" s="59">
+        <v>1</v>
+      </c>
+      <c r="B4" s="59">
+        <v>1</v>
+      </c>
+      <c r="C4" s="59">
+        <v>30</v>
+      </c>
+      <c r="D4" s="59">
+        <v>1</v>
+      </c>
+      <c r="E4" s="59" t="str">
+        <f>IF(D4=0,"Compra","Venda")</f>
+        <v>Venda</v>
+      </c>
+      <c r="F4" s="75">
+        <v>2404</v>
+      </c>
+      <c r="G4" s="75">
+        <f t="shared" ref="G4:G6" si="0">G3+IF(D4=0,F4,-F4)</f>
+        <v>1.8279999999999745</v>
+      </c>
+      <c r="H4" s="59">
+        <v>5</v>
+      </c>
+      <c r="J4" s="68">
+        <v>41971</v>
+      </c>
+      <c r="K4" s="73">
+        <v>19.354099999999999</v>
+      </c>
+      <c r="L4" s="73">
+        <v>18.524504991680502</v>
+      </c>
+      <c r="N4" s="59" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
+      <c r="A5" s="59">
+        <v>1</v>
+      </c>
+      <c r="B5" s="59">
+        <v>1</v>
+      </c>
+      <c r="C5" s="59">
+        <v>92</v>
+      </c>
+      <c r="D5" s="59">
+        <v>0</v>
+      </c>
+      <c r="E5" s="59" t="str">
+        <f t="shared" ref="E5:E69" si="1">IF(D5=0,"Compra","Venda")</f>
+        <v>Compra</v>
+      </c>
+      <c r="F5" s="75">
+        <v>2922.36</v>
+      </c>
+      <c r="G5" s="75">
+        <f t="shared" si="0"/>
+        <v>2924.1880000000001</v>
+      </c>
+      <c r="H5" s="59">
+        <v>5</v>
+      </c>
+      <c r="I5" s="59">
+        <v>91</v>
+      </c>
+      <c r="J5" s="68">
+        <v>42202.719108796293</v>
+      </c>
+      <c r="K5" s="73">
+        <v>15.6417</v>
+      </c>
+      <c r="L5" s="73">
+        <v>18.393100097181701</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
+      <c r="A6" s="59">
+        <v>1</v>
+      </c>
+      <c r="B6" s="59">
+        <v>1</v>
+      </c>
+      <c r="C6" s="59">
+        <v>100</v>
+      </c>
+      <c r="D6" s="59">
+        <v>1</v>
+      </c>
+      <c r="E6" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Venda</v>
+      </c>
+      <c r="F6" s="75">
+        <v>2879.2429999999999</v>
+      </c>
+      <c r="G6" s="75">
+        <f t="shared" si="0"/>
+        <v>44.945000000000164</v>
+      </c>
+      <c r="H6" s="59">
+        <v>16</v>
+      </c>
+      <c r="J6" s="68">
+        <v>42279.463796296295</v>
+      </c>
+      <c r="K6" s="73">
+        <v>15.6441</v>
+      </c>
+      <c r="L6" s="73">
+        <v>18.063202723771401</v>
+      </c>
+      <c r="N6" s="59" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14">
+      <c r="J7" s="68"/>
+    </row>
+    <row r="8" spans="1:14">
+      <c r="A8" s="59">
+        <v>1</v>
+      </c>
+      <c r="B8" s="59">
+        <v>2</v>
+      </c>
+      <c r="C8" s="59">
+        <v>37</v>
+      </c>
+      <c r="D8" s="59">
+        <v>0</v>
+      </c>
+      <c r="E8" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Compra</v>
+      </c>
+      <c r="F8" s="75">
+        <v>76.745999999999995</v>
+      </c>
+      <c r="J8" s="68">
+        <v>41534</v>
+      </c>
+      <c r="K8" s="73">
+        <v>13.03</v>
+      </c>
+      <c r="L8" s="73">
+        <v>13.029995048601799</v>
+      </c>
+      <c r="N8" s="59" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
+      <c r="A9" s="59">
+        <v>1</v>
+      </c>
+      <c r="B9" s="59">
+        <v>2</v>
+      </c>
+      <c r="C9" s="59">
+        <v>38</v>
+      </c>
+      <c r="D9" s="59">
+        <v>1</v>
+      </c>
+      <c r="E9" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Venda</v>
+      </c>
+      <c r="F9" s="75">
+        <v>75</v>
+      </c>
+      <c r="H9" s="59">
+        <v>6</v>
+      </c>
+      <c r="J9" s="68">
+        <v>41673</v>
+      </c>
+      <c r="K9" s="73">
+        <v>13.03</v>
+      </c>
+      <c r="L9" s="73">
+        <v>12.78</v>
+      </c>
+      <c r="N9" s="59" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14">
+      <c r="A10" s="59">
+        <v>1</v>
+      </c>
+      <c r="B10" s="59">
+        <v>2</v>
+      </c>
+      <c r="C10" s="59">
+        <v>103</v>
+      </c>
+      <c r="D10" s="59">
+        <v>1</v>
+      </c>
+      <c r="E10" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Venda</v>
+      </c>
+      <c r="F10" s="75">
+        <v>1.746</v>
+      </c>
+      <c r="H10" s="59">
+        <v>6</v>
+      </c>
+      <c r="J10" s="68">
+        <v>42310.831203703703</v>
+      </c>
+      <c r="K10" s="73">
+        <v>13.03</v>
+      </c>
+      <c r="L10" s="73">
+        <v>13.6483390607101</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14">
+      <c r="A11" s="59">
+        <v>1</v>
+      </c>
+      <c r="B11" s="59">
+        <v>3</v>
+      </c>
+      <c r="C11" s="59">
+        <v>1</v>
+      </c>
+      <c r="D11" s="59">
+        <v>0</v>
+      </c>
+      <c r="E11" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Compra</v>
+      </c>
+      <c r="F11" s="75">
+        <v>325.52199999999999</v>
+      </c>
+      <c r="J11" s="68">
+        <v>41172</v>
+      </c>
+      <c r="K11" s="73">
+        <v>30.719899999999999</v>
+      </c>
+      <c r="L11" s="73">
+        <v>30.719859180024699</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14">
+      <c r="A12" s="59">
+        <v>1</v>
+      </c>
+      <c r="B12" s="59">
+        <v>3</v>
+      </c>
+      <c r="C12" s="59">
+        <v>2</v>
+      </c>
+      <c r="D12" s="59">
+        <v>0</v>
+      </c>
+      <c r="E12" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Compra</v>
+      </c>
+      <c r="F12" s="75">
+        <v>1267.6880000000001</v>
+      </c>
+      <c r="J12" s="68">
+        <v>41187</v>
+      </c>
+      <c r="K12" s="73">
+        <v>31.5535</v>
+      </c>
+      <c r="L12" s="73">
+        <v>31.5534895021487</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14">
+      <c r="A13" s="59">
+        <v>1</v>
+      </c>
+      <c r="B13" s="59">
+        <v>3</v>
+      </c>
+      <c r="C13" s="59">
+        <v>3</v>
+      </c>
+      <c r="D13" s="59">
+        <v>0</v>
+      </c>
+      <c r="E13" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Compra</v>
+      </c>
+      <c r="F13" s="75">
+        <v>522.37400000000002</v>
+      </c>
+      <c r="J13" s="68">
+        <v>41410</v>
+      </c>
+      <c r="K13" s="73">
+        <v>38.286799999999999</v>
+      </c>
+      <c r="L13" s="73">
+        <v>38.286783032846103</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14">
+      <c r="A14" s="59">
+        <v>1</v>
+      </c>
+      <c r="B14" s="59">
+        <v>3</v>
+      </c>
+      <c r="C14" s="59">
+        <v>4</v>
+      </c>
+      <c r="D14" s="59">
+        <v>1</v>
+      </c>
+      <c r="E14" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Venda</v>
+      </c>
+      <c r="F14" s="75">
+        <v>1415.5820000000001</v>
+      </c>
+      <c r="J14" s="68">
+        <v>41438</v>
+      </c>
+      <c r="K14" s="73">
+        <v>31.361799999999999</v>
+      </c>
+      <c r="L14" s="73">
+        <v>33.983393402854702</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14">
+      <c r="A15" s="59">
+        <v>1</v>
+      </c>
+      <c r="B15" s="59">
+        <v>3</v>
+      </c>
+      <c r="C15" s="59">
+        <v>5</v>
+      </c>
+      <c r="D15" s="59">
+        <v>1</v>
+      </c>
+      <c r="E15" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Venda</v>
+      </c>
+      <c r="F15" s="75">
+        <v>178</v>
+      </c>
+      <c r="J15" s="68">
+        <v>41492</v>
+      </c>
+      <c r="K15" s="73">
+        <v>31.567599999999999</v>
+      </c>
+      <c r="L15" s="73">
+        <v>33.896398876404497</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14">
+      <c r="A16" s="59">
+        <v>1</v>
+      </c>
+      <c r="B16" s="59">
+        <v>3</v>
+      </c>
+      <c r="C16" s="59">
+        <v>6</v>
+      </c>
+      <c r="D16" s="59">
+        <v>1</v>
+      </c>
+      <c r="E16" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Venda</v>
+      </c>
+      <c r="F16" s="75">
+        <v>522.00199999999995</v>
+      </c>
+      <c r="J16" s="68">
+        <v>41506</v>
+      </c>
+      <c r="K16" s="73">
+        <v>38.286799999999999</v>
+      </c>
+      <c r="L16" s="73">
+        <v>32.470297048670297</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14">
+      <c r="A17" s="59">
+        <v>1</v>
+      </c>
+      <c r="B17" s="59">
+        <v>3</v>
+      </c>
+      <c r="C17" s="59">
+        <v>41</v>
+      </c>
+      <c r="D17" s="59">
+        <v>0</v>
+      </c>
+      <c r="E17" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Compra</v>
+      </c>
+      <c r="F17" s="75">
+        <v>174.22900000000001</v>
+      </c>
+      <c r="H17" s="59">
+        <v>6</v>
+      </c>
+      <c r="I17" s="59">
+        <v>40</v>
+      </c>
+      <c r="J17" s="68">
+        <v>42047.000011574077</v>
+      </c>
+      <c r="K17" s="73">
+        <v>21.561399999999999</v>
+      </c>
+      <c r="L17" s="73">
+        <v>39.4291363665061</v>
+      </c>
+      <c r="N17" s="59" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14">
+      <c r="A18" s="59">
+        <v>1</v>
+      </c>
+      <c r="B18" s="59">
+        <v>3</v>
+      </c>
+      <c r="C18" s="59">
+        <v>95</v>
+      </c>
+      <c r="D18" s="59">
+        <v>1</v>
+      </c>
+      <c r="E18" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Venda</v>
+      </c>
+      <c r="F18" s="75">
+        <v>150</v>
+      </c>
+      <c r="H18" s="59">
+        <v>6</v>
+      </c>
+      <c r="J18" s="68">
+        <v>42207.759375000001</v>
+      </c>
+      <c r="K18" s="73">
+        <v>21.561399999999999</v>
+      </c>
+      <c r="L18" s="73">
+        <v>39.577666666666602</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14">
+      <c r="A19" s="59">
+        <v>1</v>
+      </c>
+      <c r="B19" s="59">
+        <v>4</v>
+      </c>
+      <c r="C19" s="59">
+        <v>11</v>
+      </c>
+      <c r="D19" s="59">
+        <v>0</v>
+      </c>
+      <c r="E19" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Compra</v>
+      </c>
+      <c r="F19" s="75">
+        <v>28.28</v>
+      </c>
+      <c r="J19" s="68">
+        <v>41554</v>
+      </c>
+      <c r="K19" s="73">
+        <v>35.357100000000003</v>
+      </c>
+      <c r="L19" s="73">
+        <v>35.357142857142797</v>
+      </c>
+      <c r="N19" s="59" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14">
+      <c r="A20" s="59">
+        <v>1</v>
+      </c>
+      <c r="B20" s="59">
+        <v>4</v>
+      </c>
+      <c r="C20" s="59">
+        <v>12</v>
+      </c>
+      <c r="D20" s="59">
+        <v>0</v>
+      </c>
+      <c r="E20" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Compra</v>
+      </c>
+      <c r="F20" s="75">
+        <v>134.86000000000001</v>
+      </c>
+      <c r="J20" s="68">
+        <v>41565</v>
+      </c>
+      <c r="K20" s="73">
+        <v>37.076300000000003</v>
+      </c>
+      <c r="L20" s="73">
+        <v>37.076301349547599</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14">
+      <c r="A21" s="59">
+        <v>1</v>
+      </c>
+      <c r="B21" s="59">
+        <v>4</v>
+      </c>
+      <c r="C21" s="59">
+        <v>13</v>
+      </c>
+      <c r="D21" s="59">
+        <v>1</v>
+      </c>
+      <c r="E21" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Venda</v>
+      </c>
+      <c r="F21" s="75">
+        <v>160</v>
+      </c>
+      <c r="J21" s="68">
+        <v>41639</v>
+      </c>
+      <c r="K21" s="73">
+        <v>36.772399999999998</v>
+      </c>
+      <c r="L21" s="73">
+        <v>30.947749999999999</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14">
+      <c r="A22" s="59">
+        <v>1</v>
+      </c>
+      <c r="B22" s="59">
+        <v>5</v>
+      </c>
+      <c r="C22" s="59">
+        <v>26</v>
+      </c>
+      <c r="D22" s="59">
+        <v>0</v>
+      </c>
+      <c r="E22" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Compra</v>
+      </c>
+      <c r="F22" s="75">
+        <v>249.34710000000001</v>
+      </c>
+      <c r="H22" s="59">
+        <v>11</v>
+      </c>
+      <c r="I22" s="59">
+        <v>25</v>
+      </c>
+      <c r="J22" s="68">
+        <v>41439.000011574077</v>
+      </c>
+      <c r="K22" s="73">
+        <v>182.98320000000001</v>
+      </c>
+      <c r="L22" s="73">
+        <v>139.70998660100699</v>
+      </c>
+      <c r="N22" s="59" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14">
+      <c r="A23" s="59">
+        <v>1</v>
+      </c>
+      <c r="B23" s="59">
+        <v>5</v>
+      </c>
+      <c r="C23" s="59">
+        <v>28</v>
+      </c>
+      <c r="D23" s="59">
+        <v>1</v>
+      </c>
+      <c r="E23" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Venda</v>
+      </c>
+      <c r="F23" s="75">
+        <v>249</v>
+      </c>
+      <c r="H23" s="59">
+        <v>1</v>
+      </c>
+      <c r="J23" s="68">
+        <v>41794</v>
+      </c>
+      <c r="K23" s="73">
+        <v>182.98320000000001</v>
+      </c>
+      <c r="L23" s="73">
+        <v>172.04</v>
+      </c>
+      <c r="N23" s="59" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14">
+      <c r="A24" s="59">
+        <v>1</v>
+      </c>
+      <c r="B24" s="59">
+        <v>5</v>
+      </c>
+      <c r="C24" s="59">
+        <v>31</v>
+      </c>
+      <c r="D24" s="59">
+        <v>0</v>
+      </c>
+      <c r="E24" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Compra</v>
+      </c>
+      <c r="F24" s="75">
+        <v>264.18049999999999</v>
+      </c>
+      <c r="H24" s="59">
+        <v>1</v>
+      </c>
+      <c r="I24" s="59">
+        <v>30</v>
+      </c>
+      <c r="J24" s="68">
+        <v>41976</v>
+      </c>
+      <c r="K24" s="73">
+        <v>176.11920000000001</v>
+      </c>
+      <c r="L24" s="73">
+        <v>168.57001179118001</v>
+      </c>
+      <c r="N24" s="59" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14">
+      <c r="A25" s="59">
+        <v>1</v>
+      </c>
+      <c r="B25" s="59">
+        <v>5</v>
+      </c>
+      <c r="C25" s="59">
+        <v>91</v>
+      </c>
+      <c r="D25" s="59">
+        <v>1</v>
+      </c>
+      <c r="E25" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Venda</v>
+      </c>
+      <c r="F25" s="75">
+        <v>259.52999999999997</v>
+      </c>
+      <c r="H25" s="59">
+        <v>1</v>
+      </c>
+      <c r="J25" s="68">
+        <v>42201.719108796293</v>
+      </c>
+      <c r="K25" s="73">
+        <v>176.1284</v>
+      </c>
+      <c r="L25" s="73">
+        <v>207.11000655030199</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14">
+      <c r="A26" s="59">
+        <v>1</v>
+      </c>
+      <c r="B26" s="59">
+        <v>6</v>
+      </c>
+      <c r="C26" s="59">
+        <v>7</v>
+      </c>
+      <c r="D26" s="59">
+        <v>0</v>
+      </c>
+      <c r="E26" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Compra</v>
+      </c>
+      <c r="F26" s="75">
+        <v>24.091999999999999</v>
+      </c>
+      <c r="J26" s="68">
+        <v>41492.000011574077</v>
+      </c>
+      <c r="K26" s="73">
+        <v>250.44120000000001</v>
+      </c>
+      <c r="L26" s="73">
+        <v>250.44122530300501</v>
+      </c>
+      <c r="N26" s="59" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14">
+      <c r="A27" s="59">
+        <v>1</v>
+      </c>
+      <c r="B27" s="59">
+        <v>6</v>
+      </c>
+      <c r="C27" s="59">
+        <v>39</v>
+      </c>
+      <c r="D27" s="59">
+        <v>0</v>
+      </c>
+      <c r="E27" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Compra</v>
+      </c>
+      <c r="F27" s="75">
+        <v>3.1440000000000001</v>
+      </c>
+      <c r="H27" s="59">
+        <v>2</v>
+      </c>
+      <c r="I27" s="59">
+        <v>38</v>
+      </c>
+      <c r="J27" s="68">
+        <v>41673.000011574077</v>
+      </c>
+      <c r="K27" s="73">
+        <v>310.83019999999999</v>
+      </c>
+      <c r="L27" s="73">
+        <v>304.86641221373998</v>
+      </c>
+      <c r="N27" s="59" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14">
+      <c r="A28" s="59">
+        <v>1</v>
+      </c>
+      <c r="B28" s="59">
+        <v>6</v>
+      </c>
+      <c r="C28" s="59">
+        <v>40</v>
+      </c>
+      <c r="D28" s="59">
+        <v>1</v>
+      </c>
+      <c r="E28" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Venda</v>
+      </c>
+      <c r="F28" s="75">
+        <v>15</v>
+      </c>
+      <c r="H28" s="59">
+        <v>3</v>
+      </c>
+      <c r="J28" s="68">
+        <v>42047</v>
+      </c>
+      <c r="K28" s="73">
+        <v>250.44120000000001</v>
+      </c>
+      <c r="L28" s="73">
+        <v>457.97993333333301</v>
+      </c>
+      <c r="N28" s="59" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14">
+      <c r="A29" s="59">
+        <v>1</v>
+      </c>
+      <c r="B29" s="59">
+        <v>6</v>
+      </c>
+      <c r="C29" s="59">
+        <v>96</v>
+      </c>
+      <c r="D29" s="59">
+        <v>0</v>
+      </c>
+      <c r="E29" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Compra</v>
+      </c>
+      <c r="F29" s="75">
+        <v>10.042999999999999</v>
+      </c>
+      <c r="H29" s="59">
+        <v>3</v>
+      </c>
+      <c r="I29" s="59">
+        <v>95</v>
+      </c>
+      <c r="J29" s="68">
+        <v>42208.759375000001</v>
+      </c>
+      <c r="K29" s="73">
+        <v>322.03620000000001</v>
+      </c>
+      <c r="L29" s="73">
+        <v>591.12317036742002</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14">
+      <c r="A30" s="59">
+        <v>1</v>
+      </c>
+      <c r="B30" s="59">
+        <v>6</v>
+      </c>
+      <c r="C30" s="59">
+        <v>104</v>
+      </c>
+      <c r="D30" s="59">
+        <v>0</v>
+      </c>
+      <c r="E30" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Compra</v>
+      </c>
+      <c r="F30" s="75">
+        <v>4.7E-2</v>
+      </c>
+      <c r="H30" s="59">
+        <v>2</v>
+      </c>
+      <c r="I30" s="59">
+        <v>103</v>
+      </c>
+      <c r="J30" s="68">
+        <v>42311.831203703703</v>
+      </c>
+      <c r="K30" s="73">
+        <v>484.05059999999997</v>
+      </c>
+      <c r="L30" s="73">
+        <v>507.02127659574398</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14">
+      <c r="A31" s="59">
+        <v>1</v>
+      </c>
+      <c r="B31" s="59">
+        <v>7</v>
+      </c>
+      <c r="C31" s="59">
+        <v>79</v>
+      </c>
+      <c r="D31" s="59">
+        <v>0</v>
+      </c>
+      <c r="E31" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Compra</v>
+      </c>
+      <c r="F31" s="75">
+        <v>925</v>
+      </c>
+      <c r="J31" s="68">
+        <v>41711</v>
+      </c>
+      <c r="K31" s="73">
+        <v>10.824999999999999</v>
+      </c>
+      <c r="L31" s="73">
+        <v>10.824999999999999</v>
+      </c>
+      <c r="M31" s="71">
+        <v>15.06</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14">
+      <c r="A32" s="59">
+        <v>1</v>
+      </c>
+      <c r="B32" s="59">
+        <v>7</v>
+      </c>
+      <c r="C32" s="59">
+        <v>80</v>
+      </c>
+      <c r="D32" s="59">
+        <v>1</v>
+      </c>
+      <c r="E32" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Venda</v>
+      </c>
+      <c r="F32" s="75">
+        <v>925</v>
+      </c>
+      <c r="J32" s="68">
+        <v>41717</v>
+      </c>
+      <c r="K32" s="73">
+        <v>10.824999999999999</v>
+      </c>
+      <c r="L32" s="73">
+        <v>11.05</v>
+      </c>
+      <c r="M32" s="71">
+        <v>25.32</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14">
+      <c r="A33" s="59">
+        <v>1</v>
+      </c>
+      <c r="B33" s="59">
+        <v>7</v>
+      </c>
+      <c r="C33" s="59">
+        <v>81</v>
+      </c>
+      <c r="D33" s="59">
+        <v>0</v>
+      </c>
+      <c r="E33" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Compra</v>
+      </c>
+      <c r="F33" s="75">
+        <v>929</v>
+      </c>
+      <c r="J33" s="68">
+        <v>41830</v>
+      </c>
+      <c r="K33" s="73">
+        <v>10.74</v>
+      </c>
+      <c r="L33" s="73">
+        <v>10.739999999999901</v>
+      </c>
+      <c r="M33" s="71">
+        <v>15.06</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14">
+      <c r="A34" s="59">
+        <v>1</v>
+      </c>
+      <c r="B34" s="59">
+        <v>7</v>
+      </c>
+      <c r="C34" s="59">
+        <v>82</v>
+      </c>
+      <c r="D34" s="59">
+        <v>1</v>
+      </c>
+      <c r="E34" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Venda</v>
+      </c>
+      <c r="F34" s="75">
+        <v>929</v>
+      </c>
+      <c r="J34" s="68">
+        <v>41877</v>
+      </c>
+      <c r="K34" s="73">
+        <v>10.74</v>
+      </c>
+      <c r="L34" s="73">
+        <v>10.98</v>
+      </c>
+      <c r="M34" s="71">
+        <v>15.09</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14">
+      <c r="A35" s="59">
+        <v>1</v>
+      </c>
+      <c r="B35" s="59">
+        <v>7</v>
+      </c>
+      <c r="C35" s="59">
+        <v>83</v>
+      </c>
+      <c r="D35" s="59">
+        <v>0</v>
+      </c>
+      <c r="E35" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Compra</v>
+      </c>
+      <c r="F35" s="75">
+        <v>5386</v>
+      </c>
+      <c r="J35" s="68">
+        <v>41984</v>
+      </c>
+      <c r="K35" s="73">
+        <v>9.2676999999999996</v>
+      </c>
+      <c r="L35" s="73">
+        <v>9.2677385815076097</v>
+      </c>
+      <c r="M35" s="71">
+        <v>20.14</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14">
+      <c r="A36" s="59">
+        <v>1</v>
+      </c>
+      <c r="B36" s="59">
+        <v>7</v>
+      </c>
+      <c r="C36" s="59">
+        <v>84</v>
+      </c>
+      <c r="D36" s="59">
+        <v>1</v>
+      </c>
+      <c r="E36" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Venda</v>
+      </c>
+      <c r="F36" s="75">
+        <v>5386</v>
+      </c>
+      <c r="J36" s="68">
+        <v>42047.000023148146</v>
+      </c>
+      <c r="K36" s="73">
+        <v>9.2676999999999996</v>
+      </c>
+      <c r="L36" s="73">
+        <v>9.0449999999999999</v>
+      </c>
+      <c r="M36" s="71">
+        <v>20.03</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14">
+      <c r="A37" s="59">
+        <v>1</v>
+      </c>
+      <c r="B37" s="59">
+        <v>7</v>
+      </c>
+      <c r="C37" s="59">
+        <v>94</v>
+      </c>
+      <c r="D37" s="59">
+        <v>0</v>
+      </c>
+      <c r="E37" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Compra</v>
+      </c>
+      <c r="F37" s="75">
+        <v>6415</v>
+      </c>
+      <c r="J37" s="68">
+        <v>42212.556203703702</v>
+      </c>
+      <c r="K37" s="73">
+        <v>7.7939999999999996</v>
+      </c>
+      <c r="L37" s="73">
+        <v>7.7939999999999996</v>
+      </c>
+      <c r="M37" s="71">
+        <v>20.149999999999999</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14">
+      <c r="A38" s="59">
+        <v>1</v>
+      </c>
+      <c r="B38" s="59">
+        <v>7</v>
+      </c>
+      <c r="C38" s="59">
+        <v>97</v>
+      </c>
+      <c r="D38" s="59">
+        <v>1</v>
+      </c>
+      <c r="E38" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Venda</v>
+      </c>
+      <c r="F38" s="75">
+        <v>6415</v>
+      </c>
+      <c r="J38" s="68">
+        <v>42214.282905092594</v>
+      </c>
+      <c r="K38" s="73">
+        <v>7.7939999999999996</v>
+      </c>
+      <c r="L38" s="73">
+        <v>8.19</v>
+      </c>
+      <c r="M38" s="71">
+        <v>20.399999999999999</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14">
+      <c r="A39" s="59">
+        <v>1</v>
+      </c>
+      <c r="B39" s="59">
+        <v>7</v>
+      </c>
+      <c r="C39" s="59">
+        <v>138</v>
+      </c>
+      <c r="D39" s="59">
+        <v>5</v>
+      </c>
+      <c r="E39" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Venda</v>
+      </c>
+      <c r="F39" s="75">
+        <v>1581</v>
+      </c>
+      <c r="J39" s="68">
+        <v>42822.416643518518</v>
+      </c>
+      <c r="K39" s="73">
+        <v>7.5910000000000002</v>
+      </c>
+      <c r="L39" s="73">
+        <v>7.5910000000000002</v>
+      </c>
+      <c r="M39" s="71">
+        <v>15.15</v>
+      </c>
+      <c r="N39" s="59" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14">
+      <c r="A40" s="59">
+        <v>1</v>
+      </c>
+      <c r="B40" s="59">
+        <v>7</v>
+      </c>
+      <c r="C40" s="59">
+        <v>151</v>
+      </c>
+      <c r="D40" s="59">
+        <v>0</v>
+      </c>
+      <c r="E40" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Compra</v>
+      </c>
+      <c r="F40" s="75">
+        <v>527</v>
+      </c>
+      <c r="J40" s="68">
+        <v>42822.416655092595</v>
+      </c>
+      <c r="K40" s="73">
+        <v>22.773</v>
+      </c>
+      <c r="L40" s="73">
+        <v>22.773</v>
+      </c>
+      <c r="M40" s="71">
+        <v>15.15</v>
+      </c>
+      <c r="N40" s="59" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14">
+      <c r="A41" s="59">
+        <v>1</v>
+      </c>
+      <c r="B41" s="59">
+        <v>7</v>
+      </c>
+      <c r="C41" s="59">
+        <v>165</v>
+      </c>
+      <c r="D41" s="59">
+        <v>1</v>
+      </c>
+      <c r="E41" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Venda</v>
+      </c>
+      <c r="F41" s="75">
+        <v>527</v>
+      </c>
+      <c r="J41" s="68">
+        <v>43236.344560185185</v>
+      </c>
+      <c r="K41" s="73">
+        <v>22.773</v>
+      </c>
+      <c r="L41" s="73">
+        <v>30.416039999999999</v>
+      </c>
+      <c r="M41" s="71">
+        <v>27.45</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14">
+      <c r="A42" s="59">
+        <v>1</v>
+      </c>
+      <c r="B42" s="59">
+        <v>8</v>
+      </c>
+      <c r="C42" s="59">
+        <v>78</v>
+      </c>
+      <c r="D42" s="59">
+        <v>0</v>
+      </c>
+      <c r="E42" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Compra</v>
+      </c>
+      <c r="F42" s="75">
+        <v>7743</v>
+      </c>
+      <c r="J42" s="68">
+        <v>42058</v>
+      </c>
+      <c r="K42" s="73">
+        <v>6.4550000000000001</v>
+      </c>
+      <c r="L42" s="73">
+        <v>6.4550000000000001</v>
+      </c>
+      <c r="M42" s="71">
+        <v>20.18</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14">
+      <c r="A43" s="59">
+        <v>1</v>
+      </c>
+      <c r="B43" s="59">
+        <v>8</v>
+      </c>
+      <c r="C43" s="59">
+        <v>86</v>
+      </c>
+      <c r="D43" s="59">
+        <v>0</v>
+      </c>
+      <c r="E43" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Compra</v>
+      </c>
+      <c r="F43" s="75">
+        <v>168</v>
+      </c>
+      <c r="J43" s="68">
+        <v>42123.703634259262</v>
+      </c>
+      <c r="K43" s="73">
+        <v>0</v>
+      </c>
+      <c r="L43" s="73">
+        <v>0</v>
+      </c>
+      <c r="N43" s="59" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14">
+      <c r="A44" s="59">
+        <v>1</v>
+      </c>
+      <c r="B44" s="59">
+        <v>8</v>
+      </c>
+      <c r="C44" s="59">
+        <v>88</v>
+      </c>
+      <c r="D44" s="59">
+        <v>2</v>
+      </c>
+      <c r="E44" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Venda</v>
+      </c>
+      <c r="F44" s="75">
+        <v>0</v>
+      </c>
+      <c r="J44" s="68">
+        <v>42117.864814814813</v>
+      </c>
+      <c r="L44" s="73">
+        <v>2.27</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14">
+      <c r="A45" s="59">
+        <v>1</v>
+      </c>
+      <c r="B45" s="59">
+        <v>8</v>
+      </c>
+      <c r="C45" s="59">
+        <v>89</v>
+      </c>
+      <c r="D45" s="59">
+        <v>1</v>
+      </c>
+      <c r="E45" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Venda</v>
+      </c>
+      <c r="F45" s="75">
+        <v>7911</v>
+      </c>
+      <c r="J45" s="68">
+        <v>42200.864814814813</v>
+      </c>
+      <c r="K45" s="73">
+        <v>6.3178999999999998</v>
+      </c>
+      <c r="L45" s="73">
+        <v>6.63</v>
+      </c>
+      <c r="M45" s="71">
+        <v>20.38</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14">
+      <c r="A46" s="59">
+        <v>1</v>
+      </c>
+      <c r="B46" s="59">
+        <v>9</v>
+      </c>
+      <c r="C46" s="59">
+        <v>43</v>
+      </c>
+      <c r="D46" s="59">
+        <v>0</v>
+      </c>
+      <c r="E46" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Compra</v>
+      </c>
+      <c r="F46" s="75">
+        <v>60</v>
+      </c>
+      <c r="J46" s="68">
+        <v>36850</v>
+      </c>
+      <c r="K46" s="73">
+        <v>20.100000000000001</v>
+      </c>
+      <c r="L46" s="73">
+        <v>20.100000000000001</v>
+      </c>
+      <c r="M46" s="71">
+        <v>2.5299999999999998</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14">
+      <c r="A47" s="59">
+        <v>1</v>
+      </c>
+      <c r="B47" s="59">
+        <v>9</v>
+      </c>
+      <c r="C47" s="59">
+        <v>45</v>
+      </c>
+      <c r="D47" s="59">
+        <v>2</v>
+      </c>
+      <c r="E47" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Venda</v>
+      </c>
+      <c r="F47" s="75">
+        <v>0</v>
+      </c>
+      <c r="J47" s="68">
+        <v>36909</v>
+      </c>
+      <c r="L47" s="73">
+        <v>3.54</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14">
+      <c r="A48" s="59">
+        <v>1</v>
+      </c>
+      <c r="B48" s="59">
+        <v>9</v>
+      </c>
+      <c r="C48" s="59">
+        <v>46</v>
+      </c>
+      <c r="D48" s="59">
+        <v>0</v>
+      </c>
+      <c r="E48" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Compra</v>
+      </c>
+      <c r="F48" s="75">
+        <v>1</v>
+      </c>
+      <c r="J48" s="68">
+        <v>36910</v>
+      </c>
+      <c r="K48" s="73">
+        <v>3.25</v>
+      </c>
+      <c r="L48" s="73">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="49" spans="1:14">
+      <c r="A49" s="59">
+        <v>1</v>
+      </c>
+      <c r="B49" s="59">
+        <v>9</v>
+      </c>
+      <c r="C49" s="59">
+        <v>47</v>
+      </c>
+      <c r="D49" s="59">
+        <v>2</v>
+      </c>
+      <c r="E49" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Venda</v>
+      </c>
+      <c r="F49" s="75">
+        <v>0</v>
+      </c>
+      <c r="J49" s="68">
+        <v>36969</v>
+      </c>
+      <c r="L49" s="73">
+        <v>3.61</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14">
+      <c r="A50" s="59">
+        <v>1</v>
+      </c>
+      <c r="B50" s="59">
+        <v>9</v>
+      </c>
+      <c r="C50" s="59">
+        <v>48</v>
+      </c>
+      <c r="D50" s="59">
+        <v>2</v>
+      </c>
+      <c r="E50" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Venda</v>
+      </c>
+      <c r="F50" s="75">
+        <v>0</v>
+      </c>
+      <c r="J50" s="68">
+        <v>36970</v>
+      </c>
+      <c r="L50" s="73">
+        <v>17.91</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14">
+      <c r="A51" s="59">
+        <v>1</v>
+      </c>
+      <c r="B51" s="59">
+        <v>9</v>
+      </c>
+      <c r="C51" s="59">
+        <v>49</v>
+      </c>
+      <c r="D51" s="59">
+        <v>0</v>
+      </c>
+      <c r="E51" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Compra</v>
+      </c>
+      <c r="F51" s="75">
+        <v>1</v>
+      </c>
+      <c r="J51" s="68">
+        <v>36970.000011574077</v>
+      </c>
+      <c r="K51" s="73">
+        <v>3.25</v>
+      </c>
+      <c r="L51" s="73">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14">
+      <c r="A52" s="59">
+        <v>1</v>
+      </c>
+      <c r="B52" s="59">
+        <v>9</v>
+      </c>
+      <c r="C52" s="59">
+        <v>50</v>
+      </c>
+      <c r="D52" s="59">
+        <v>2</v>
+      </c>
+      <c r="E52" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Venda</v>
+      </c>
+      <c r="F52" s="75">
+        <v>0</v>
+      </c>
+      <c r="J52" s="68">
+        <v>37294</v>
+      </c>
+      <c r="L52" s="73">
+        <v>2.31</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14">
+      <c r="A53" s="59">
+        <v>1</v>
+      </c>
+      <c r="B53" s="59">
+        <v>9</v>
+      </c>
+      <c r="C53" s="59">
+        <v>51</v>
+      </c>
+      <c r="D53" s="59">
+        <v>0</v>
+      </c>
+      <c r="E53" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Compra</v>
+      </c>
+      <c r="F53" s="75">
+        <v>1</v>
+      </c>
+      <c r="J53" s="68">
+        <v>37295</v>
+      </c>
+      <c r="K53" s="73">
+        <v>3.25</v>
+      </c>
+      <c r="L53" s="73">
+        <v>3.25</v>
+      </c>
+      <c r="M53" s="71">
+        <v>9.07</v>
+      </c>
+      <c r="N53" s="59" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14">
+      <c r="A54" s="59">
+        <v>1</v>
+      </c>
+      <c r="B54" s="59">
+        <v>9</v>
+      </c>
+      <c r="C54" s="59">
+        <v>52</v>
+      </c>
+      <c r="D54" s="59">
+        <v>2</v>
+      </c>
+      <c r="E54" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Venda</v>
+      </c>
+      <c r="F54" s="75">
+        <v>0</v>
+      </c>
+      <c r="J54" s="68">
+        <v>37302</v>
+      </c>
+      <c r="L54" s="73">
+        <v>16.02</v>
+      </c>
+    </row>
+    <row r="55" spans="1:14">
+      <c r="A55" s="59">
+        <v>1</v>
+      </c>
+      <c r="B55" s="59">
+        <v>9</v>
+      </c>
+      <c r="C55" s="59">
+        <v>53</v>
+      </c>
+      <c r="D55" s="59">
+        <v>0</v>
+      </c>
+      <c r="E55" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Compra</v>
+      </c>
+      <c r="F55" s="75">
+        <v>1</v>
+      </c>
+      <c r="J55" s="68">
+        <v>37351</v>
+      </c>
+      <c r="K55" s="73">
+        <v>3.25</v>
+      </c>
+      <c r="L55" s="73">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14">
+      <c r="A56" s="59">
+        <v>1</v>
+      </c>
+      <c r="B56" s="59">
+        <v>9</v>
+      </c>
+      <c r="C56" s="59">
+        <v>54</v>
+      </c>
+      <c r="D56" s="59">
+        <v>2</v>
+      </c>
+      <c r="E56" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Venda</v>
+      </c>
+      <c r="F56" s="75">
+        <v>0</v>
+      </c>
+      <c r="J56" s="68">
+        <v>37662</v>
+      </c>
+      <c r="L56" s="73">
+        <v>0.94</v>
+      </c>
+    </row>
+    <row r="57" spans="1:14">
+      <c r="A57" s="59">
+        <v>1</v>
+      </c>
+      <c r="B57" s="59">
+        <v>9</v>
+      </c>
+      <c r="C57" s="59">
+        <v>55</v>
+      </c>
+      <c r="D57" s="59">
+        <v>0</v>
+      </c>
+      <c r="E57" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Compra</v>
+      </c>
+      <c r="F57" s="75">
+        <v>1</v>
+      </c>
+      <c r="J57" s="68">
+        <v>37667</v>
+      </c>
+      <c r="K57" s="73">
+        <v>3.25</v>
+      </c>
+      <c r="L57" s="73">
+        <v>3.25</v>
+      </c>
+      <c r="M57" s="71">
+        <v>9.2799999999999994</v>
+      </c>
+      <c r="N57" s="59" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="58" spans="1:14">
+      <c r="A58" s="59">
+        <v>1</v>
+      </c>
+      <c r="B58" s="59">
+        <v>9</v>
+      </c>
+      <c r="C58" s="59">
+        <v>56</v>
+      </c>
+      <c r="D58" s="59">
+        <v>2</v>
+      </c>
+      <c r="E58" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Venda</v>
+      </c>
+      <c r="F58" s="75">
+        <v>0</v>
+      </c>
+      <c r="J58" s="68">
+        <v>37705</v>
+      </c>
+      <c r="L58" s="73">
+        <v>1.1100000000000001</v>
+      </c>
+    </row>
+    <row r="59" spans="1:14">
+      <c r="A59" s="59">
+        <v>1</v>
+      </c>
+      <c r="B59" s="59">
+        <v>9</v>
+      </c>
+      <c r="C59" s="59">
+        <v>57</v>
+      </c>
+      <c r="D59" s="59">
+        <v>2</v>
+      </c>
+      <c r="E59" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Venda</v>
+      </c>
+      <c r="F59" s="75">
+        <v>0</v>
+      </c>
+      <c r="J59" s="68">
+        <v>37805</v>
+      </c>
+      <c r="L59" s="73">
+        <v>7.68</v>
+      </c>
+    </row>
+    <row r="60" spans="1:14">
+      <c r="A60" s="59">
+        <v>1</v>
+      </c>
+      <c r="B60" s="59">
+        <v>9</v>
+      </c>
+      <c r="C60" s="59">
+        <v>58</v>
+      </c>
+      <c r="D60" s="59">
+        <v>0</v>
+      </c>
+      <c r="E60" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Compra</v>
+      </c>
+      <c r="F60" s="75">
+        <v>1</v>
+      </c>
+      <c r="J60" s="68">
+        <v>37712</v>
+      </c>
+      <c r="K60" s="73">
+        <v>3</v>
+      </c>
+      <c r="L60" s="73">
+        <v>3</v>
+      </c>
+      <c r="M60" s="71">
+        <v>4.6399999999999997</v>
+      </c>
+    </row>
+    <row r="61" spans="1:14">
+      <c r="A61" s="59">
+        <v>1</v>
+      </c>
+      <c r="B61" s="59">
+        <v>9</v>
+      </c>
+      <c r="C61" s="59">
+        <v>59</v>
+      </c>
+      <c r="D61" s="59">
+        <v>2</v>
+      </c>
+      <c r="E61" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Venda</v>
+      </c>
+      <c r="F61" s="75">
+        <v>0</v>
+      </c>
+      <c r="J61" s="68">
+        <v>37909</v>
+      </c>
+      <c r="L61" s="73">
+        <v>7.02</v>
+      </c>
+    </row>
+    <row r="62" spans="1:14">
+      <c r="A62" s="59">
+        <v>1</v>
+      </c>
+      <c r="B62" s="59">
+        <v>9</v>
+      </c>
+      <c r="C62" s="59">
+        <v>60</v>
+      </c>
+      <c r="D62" s="59">
+        <v>2</v>
+      </c>
+      <c r="E62" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Venda</v>
+      </c>
+      <c r="F62" s="75">
+        <v>0</v>
+      </c>
+      <c r="J62" s="68">
+        <v>38303</v>
+      </c>
+      <c r="L62" s="73">
+        <v>12.04</v>
+      </c>
+    </row>
+    <row r="63" spans="1:14">
+      <c r="A63" s="59">
+        <v>1</v>
+      </c>
+      <c r="B63" s="59">
+        <v>9</v>
+      </c>
+      <c r="C63" s="59">
+        <v>61</v>
+      </c>
+      <c r="D63" s="59">
+        <v>2</v>
+      </c>
+      <c r="E63" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Venda</v>
+      </c>
+      <c r="F63" s="75">
+        <v>0</v>
+      </c>
+      <c r="J63" s="68">
+        <v>38485</v>
+      </c>
+      <c r="L63" s="73">
+        <v>11.74</v>
+      </c>
+    </row>
+    <row r="64" spans="1:14">
+      <c r="A64" s="59">
+        <v>1</v>
+      </c>
+      <c r="B64" s="59">
+        <v>9</v>
+      </c>
+      <c r="C64" s="59">
+        <v>62</v>
+      </c>
+      <c r="D64" s="59">
+        <v>2</v>
+      </c>
+      <c r="E64" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Venda</v>
+      </c>
+      <c r="F64" s="75">
+        <v>0</v>
+      </c>
+      <c r="J64" s="68">
+        <v>38531</v>
+      </c>
+      <c r="L64" s="73">
+        <v>8.6300000000000008</v>
+      </c>
+    </row>
+    <row r="65" spans="1:14">
+      <c r="A65" s="59">
+        <v>1</v>
+      </c>
+      <c r="B65" s="59">
+        <v>9</v>
+      </c>
+      <c r="C65" s="59">
+        <v>63</v>
+      </c>
+      <c r="D65" s="59">
+        <v>0</v>
+      </c>
+      <c r="E65" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Compra</v>
+      </c>
+      <c r="F65" s="75">
+        <v>3</v>
+      </c>
+      <c r="J65" s="68">
+        <v>38531.000011574077</v>
+      </c>
+      <c r="K65" s="73">
+        <v>3.3E-3</v>
+      </c>
+      <c r="L65" s="73">
+        <v>3.3333333333333301E-3</v>
+      </c>
+      <c r="M65" s="71">
+        <v>19.05</v>
+      </c>
+      <c r="N65" s="59" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="66" spans="1:14">
+      <c r="A66" s="59">
+        <v>1</v>
+      </c>
+      <c r="B66" s="59">
+        <v>9</v>
+      </c>
+      <c r="C66" s="59">
+        <v>64</v>
+      </c>
+      <c r="D66" s="59">
+        <v>0</v>
+      </c>
+      <c r="E66" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Compra</v>
+      </c>
+      <c r="F66" s="75">
+        <v>1006</v>
+      </c>
+      <c r="J66" s="68">
+        <v>41222</v>
+      </c>
+      <c r="K66" s="73">
+        <v>9.92</v>
+      </c>
+      <c r="L66" s="73">
+        <v>9.92</v>
+      </c>
+      <c r="M66" s="71">
+        <v>14.06</v>
+      </c>
+      <c r="N66" s="59" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="67" spans="1:14">
+      <c r="A67" s="59">
+        <v>1</v>
+      </c>
+      <c r="B67" s="59">
+        <v>9</v>
+      </c>
+      <c r="C67" s="59">
+        <v>65</v>
+      </c>
+      <c r="D67" s="59">
+        <v>1</v>
+      </c>
+      <c r="E67" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Venda</v>
+      </c>
+      <c r="F67" s="75">
+        <v>69</v>
+      </c>
+      <c r="J67" s="68">
+        <v>41289</v>
+      </c>
+      <c r="K67" s="73">
+        <v>17.757400000000001</v>
+      </c>
+      <c r="L67" s="73">
+        <v>10.96</v>
+      </c>
+      <c r="M67" s="71">
+        <v>13.58</v>
+      </c>
+      <c r="N67" s="59" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="68" spans="1:14">
+      <c r="A68" s="59">
+        <v>1</v>
+      </c>
+      <c r="B68" s="59">
+        <v>9</v>
+      </c>
+      <c r="C68" s="59">
+        <v>66</v>
+      </c>
+      <c r="D68" s="59">
+        <v>1</v>
+      </c>
+      <c r="E68" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Venda</v>
+      </c>
+      <c r="F68" s="75">
+        <v>1006</v>
+      </c>
+      <c r="J68" s="68">
+        <v>41289.000011574077</v>
+      </c>
+      <c r="K68" s="73">
+        <v>9.92</v>
+      </c>
+      <c r="L68" s="73">
+        <v>10.96</v>
+      </c>
+      <c r="M68" s="71">
+        <v>16.21</v>
+      </c>
+    </row>
+    <row r="69" spans="1:14">
+      <c r="A69" s="59">
+        <v>1</v>
+      </c>
+      <c r="B69" s="59">
+        <v>9</v>
+      </c>
+      <c r="C69" s="59">
+        <v>67</v>
+      </c>
+      <c r="D69" s="59">
+        <v>0</v>
+      </c>
+      <c r="E69" s="59" t="str">
+        <f t="shared" si="1"/>
+        <v>Compra</v>
+      </c>
+      <c r="F69" s="75">
+        <v>920</v>
+      </c>
+      <c r="J69" s="68">
+        <v>41317</v>
+      </c>
+      <c r="K69" s="73">
+        <v>9.8949999999999996</v>
+      </c>
+      <c r="L69" s="73">
+        <v>9.8949999999999996</v>
+      </c>
+      <c r="M69" s="71">
+        <v>13.93</v>
+      </c>
+    </row>
+    <row r="70" spans="1:14">
+      <c r="A70" s="59">
+        <v>1</v>
+      </c>
+      <c r="B70" s="59">
+        <v>9</v>
+      </c>
+      <c r="C70" s="59">
+        <v>68</v>
+      </c>
+      <c r="D70" s="59">
+        <v>0</v>
+      </c>
+      <c r="E70" s="59" t="str">
+        <f t="shared" ref="E70:E135" si="2">IF(D70=0,"Compra","Venda")</f>
+        <v>Compra</v>
+      </c>
+      <c r="F70" s="75">
+        <v>90</v>
+      </c>
+      <c r="J70" s="68">
+        <v>41317.000011574077</v>
+      </c>
+      <c r="K70" s="73">
+        <v>9.8960000000000008</v>
+      </c>
+      <c r="L70" s="73">
+        <v>9.8959999999999901</v>
+      </c>
+      <c r="M70" s="71">
+        <v>5.71</v>
+      </c>
+    </row>
+    <row r="71" spans="1:14">
+      <c r="A71" s="59">
+        <v>1</v>
+      </c>
+      <c r="B71" s="59">
+        <v>9</v>
+      </c>
+      <c r="C71" s="59">
+        <v>69</v>
+      </c>
+      <c r="D71" s="59">
+        <v>1</v>
+      </c>
+      <c r="E71" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Venda</v>
+      </c>
+      <c r="F71" s="75">
+        <v>1010</v>
+      </c>
+      <c r="J71" s="68">
+        <v>41351</v>
+      </c>
+      <c r="K71" s="73">
+        <v>9.8950999999999993</v>
+      </c>
+      <c r="L71" s="73">
+        <v>11.2</v>
+      </c>
+      <c r="M71" s="71">
+        <v>16.25</v>
+      </c>
+    </row>
+    <row r="72" spans="1:14">
+      <c r="A72" s="59">
+        <v>1</v>
+      </c>
+      <c r="B72" s="59">
+        <v>9</v>
+      </c>
+      <c r="C72" s="59">
+        <v>70</v>
+      </c>
+      <c r="D72" s="59">
+        <v>0</v>
+      </c>
+      <c r="E72" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F72" s="75">
+        <v>2008</v>
+      </c>
+      <c r="J72" s="68">
+        <v>41445</v>
+      </c>
+      <c r="K72" s="73">
+        <v>9.9209999999999994</v>
+      </c>
+      <c r="L72" s="73">
+        <v>9.9210009960159304</v>
+      </c>
+      <c r="M72" s="71">
+        <v>15.51</v>
+      </c>
+    </row>
+    <row r="73" spans="1:14">
+      <c r="A73" s="59">
+        <v>1</v>
+      </c>
+      <c r="B73" s="59">
+        <v>9</v>
+      </c>
+      <c r="C73" s="59">
+        <v>71</v>
+      </c>
+      <c r="D73" s="59">
+        <v>0</v>
+      </c>
+      <c r="E73" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F73" s="75">
+        <v>806</v>
+      </c>
+      <c r="J73" s="68">
+        <v>41458</v>
+      </c>
+      <c r="K73" s="73">
+        <v>9.5739999999999998</v>
+      </c>
+      <c r="L73" s="73">
+        <v>9.5739950372208398</v>
+      </c>
+      <c r="M73" s="71">
+        <v>13.73</v>
+      </c>
+    </row>
+    <row r="74" spans="1:14">
+      <c r="A74" s="59">
+        <v>1</v>
+      </c>
+      <c r="B74" s="59">
+        <v>9</v>
+      </c>
+      <c r="C74" s="59">
+        <v>72</v>
+      </c>
+      <c r="D74" s="59">
+        <v>0</v>
+      </c>
+      <c r="E74" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F74" s="75">
+        <v>1276</v>
+      </c>
+      <c r="J74" s="68">
+        <v>41458.000011574077</v>
+      </c>
+      <c r="K74" s="73">
+        <v>9.5730000000000004</v>
+      </c>
+      <c r="L74" s="73">
+        <v>9.5730015673981192</v>
+      </c>
+      <c r="M74" s="71">
+        <v>14.39</v>
+      </c>
+    </row>
+    <row r="75" spans="1:14">
+      <c r="A75" s="59">
+        <v>1</v>
+      </c>
+      <c r="B75" s="59">
+        <v>9</v>
+      </c>
+      <c r="C75" s="59">
+        <v>73</v>
+      </c>
+      <c r="D75" s="59">
+        <v>2</v>
+      </c>
+      <c r="E75" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Venda</v>
+      </c>
+      <c r="F75" s="75">
+        <v>0</v>
+      </c>
+      <c r="J75" s="68">
+        <v>41584</v>
+      </c>
+      <c r="L75" s="73">
+        <v>1431.5</v>
+      </c>
+    </row>
+    <row r="76" spans="1:14">
+      <c r="A76" s="59">
+        <v>1</v>
+      </c>
+      <c r="B76" s="59">
+        <v>9</v>
+      </c>
+      <c r="C76" s="59">
+        <v>74</v>
+      </c>
+      <c r="D76" s="59">
+        <v>0</v>
+      </c>
+      <c r="E76" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F76" s="75">
+        <v>1755</v>
+      </c>
+      <c r="J76" s="68">
+        <v>41667</v>
+      </c>
+      <c r="K76" s="73">
+        <v>11.35</v>
+      </c>
+      <c r="L76" s="73">
+        <v>11.35</v>
+      </c>
+      <c r="M76" s="71">
+        <v>16.510000000000002</v>
+      </c>
+    </row>
+    <row r="77" spans="1:14">
+      <c r="A77" s="59">
+        <v>1</v>
+      </c>
+      <c r="B77" s="59">
+        <v>9</v>
+      </c>
+      <c r="C77" s="59">
+        <v>75</v>
+      </c>
+      <c r="D77" s="59">
+        <v>2</v>
+      </c>
+      <c r="E77" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Venda</v>
+      </c>
+      <c r="F77" s="75">
+        <v>0</v>
+      </c>
+      <c r="J77" s="68">
+        <v>41766</v>
+      </c>
+      <c r="L77" s="73">
+        <v>2338</v>
+      </c>
+    </row>
+    <row r="78" spans="1:14">
+      <c r="A78" s="59">
+        <v>1</v>
+      </c>
+      <c r="B78" s="59">
+        <v>9</v>
+      </c>
+      <c r="C78" s="59">
+        <v>76</v>
+      </c>
+      <c r="D78" s="59">
+        <v>1</v>
+      </c>
+      <c r="E78" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Venda</v>
+      </c>
+      <c r="F78" s="75">
+        <v>5845</v>
+      </c>
+      <c r="J78" s="68">
+        <v>41792</v>
+      </c>
+      <c r="K78" s="73">
+        <v>10.2262</v>
+      </c>
+      <c r="L78" s="73">
+        <v>12.395000855431899</v>
+      </c>
+      <c r="M78" s="71">
+        <v>63.96</v>
+      </c>
+    </row>
+    <row r="79" spans="1:14">
+      <c r="A79" s="59">
+        <v>1</v>
+      </c>
+      <c r="B79" s="59">
+        <v>9</v>
+      </c>
+      <c r="C79" s="59">
+        <v>77</v>
+      </c>
+      <c r="D79" s="59">
+        <v>0</v>
+      </c>
+      <c r="E79" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F79" s="75">
+        <v>4388</v>
+      </c>
+      <c r="J79" s="68">
+        <v>42010</v>
+      </c>
+      <c r="K79" s="73">
+        <v>11.45</v>
+      </c>
+      <c r="L79" s="73">
+        <v>11.45</v>
+      </c>
+      <c r="M79" s="71">
+        <v>20.18</v>
+      </c>
+    </row>
+    <row r="80" spans="1:14">
+      <c r="A80" s="59">
+        <v>1</v>
+      </c>
+      <c r="B80" s="59">
+        <v>9</v>
+      </c>
+      <c r="C80" s="59">
+        <v>85</v>
+      </c>
+      <c r="D80" s="59">
+        <v>0</v>
+      </c>
+      <c r="E80" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F80" s="75">
+        <v>274</v>
+      </c>
+      <c r="J80" s="68">
+        <v>42115.562974537039</v>
+      </c>
+      <c r="K80" s="73">
+        <v>10.84</v>
+      </c>
+      <c r="L80" s="73">
+        <v>10.84</v>
+      </c>
+      <c r="N80" s="59" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="81" spans="1:14">
+      <c r="A81" s="59">
+        <v>1</v>
+      </c>
+      <c r="B81" s="59">
+        <v>9</v>
+      </c>
+      <c r="C81" s="59">
+        <v>87</v>
+      </c>
+      <c r="D81" s="59">
+        <v>2</v>
+      </c>
+      <c r="E81" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Venda</v>
+      </c>
+      <c r="F81" s="75">
+        <v>0</v>
+      </c>
+      <c r="J81" s="68">
+        <v>42136.837407407409</v>
+      </c>
+      <c r="L81" s="73">
+        <v>1864.8</v>
+      </c>
+      <c r="N81" s="59" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="82" spans="1:14">
+      <c r="A82" s="59">
+        <v>1</v>
+      </c>
+      <c r="B82" s="59">
+        <v>9</v>
+      </c>
+      <c r="C82" s="59">
+        <v>90</v>
+      </c>
+      <c r="D82" s="59">
+        <v>1</v>
+      </c>
+      <c r="E82" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Venda</v>
+      </c>
+      <c r="F82" s="75">
+        <v>4262</v>
+      </c>
+      <c r="J82" s="68">
+        <v>42200.86482638889</v>
+      </c>
+      <c r="K82" s="73">
+        <v>11.45</v>
+      </c>
+      <c r="L82" s="73">
+        <v>13.6</v>
+      </c>
+      <c r="M82" s="71">
+        <v>20.92</v>
+      </c>
+    </row>
+    <row r="83" spans="1:14">
+      <c r="A83" s="59">
+        <v>1</v>
+      </c>
+      <c r="B83" s="59">
+        <v>9</v>
+      </c>
+      <c r="C83" s="59">
+        <v>93</v>
+      </c>
+      <c r="D83" s="59">
+        <v>1</v>
+      </c>
+      <c r="E83" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Venda</v>
+      </c>
+      <c r="F83" s="75">
+        <v>400</v>
+      </c>
+      <c r="J83" s="68">
+        <v>42201.88890046296</v>
+      </c>
+      <c r="K83" s="73">
+        <v>11.0322</v>
+      </c>
+      <c r="L83" s="73">
+        <v>13.78</v>
+      </c>
+      <c r="M83" s="71">
+        <v>12.4</v>
+      </c>
+    </row>
+    <row r="84" spans="1:14">
+      <c r="A84" s="59">
+        <v>1</v>
+      </c>
+      <c r="B84" s="59">
+        <v>9</v>
+      </c>
+      <c r="C84" s="59">
+        <v>99</v>
+      </c>
+      <c r="D84" s="59">
+        <v>0</v>
+      </c>
+      <c r="E84" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F84" s="75">
+        <v>4570</v>
+      </c>
+      <c r="J84" s="68">
+        <v>42278.440972222219</v>
+      </c>
+      <c r="K84" s="73">
+        <v>10.91</v>
+      </c>
+      <c r="L84" s="73">
+        <v>10.91</v>
+      </c>
+      <c r="M84" s="71">
+        <v>20.14</v>
+      </c>
+    </row>
+    <row r="85" spans="1:14">
+      <c r="A85" s="59">
+        <v>1</v>
+      </c>
+      <c r="B85" s="59">
+        <v>9</v>
+      </c>
+      <c r="C85" s="59">
+        <v>102</v>
+      </c>
+      <c r="D85" s="59">
+        <v>1</v>
+      </c>
+      <c r="E85" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Venda</v>
+      </c>
+      <c r="F85" s="75">
+        <v>4570</v>
+      </c>
+      <c r="J85" s="68">
+        <v>42289.284166666665</v>
+      </c>
+      <c r="K85" s="73">
+        <v>10.91</v>
+      </c>
+      <c r="L85" s="73">
+        <v>11.595000000000001</v>
+      </c>
+      <c r="M85" s="71">
+        <v>20.440000000000001</v>
+      </c>
+    </row>
+    <row r="86" spans="1:14">
+      <c r="A86" s="59">
+        <v>1</v>
+      </c>
+      <c r="B86" s="59">
+        <v>9</v>
+      </c>
+      <c r="C86" s="59">
+        <v>106</v>
+      </c>
+      <c r="D86" s="59">
+        <v>0</v>
+      </c>
+      <c r="E86" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F86" s="75">
+        <v>4492</v>
+      </c>
+      <c r="J86" s="68">
+        <v>42342.482824074075</v>
+      </c>
+      <c r="K86" s="73">
+        <v>11.13</v>
+      </c>
+      <c r="L86" s="73">
+        <v>11.13</v>
+      </c>
+      <c r="M86" s="71">
+        <v>20.149999999999999</v>
+      </c>
+    </row>
+    <row r="87" spans="1:14">
+      <c r="A87" s="59">
+        <v>1</v>
+      </c>
+      <c r="B87" s="59">
+        <v>9</v>
+      </c>
+      <c r="C87" s="59">
+        <v>107</v>
+      </c>
+      <c r="D87" s="59">
+        <v>1</v>
+      </c>
+      <c r="E87" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Venda</v>
+      </c>
+      <c r="F87" s="75">
+        <v>4492</v>
+      </c>
+      <c r="J87" s="68">
+        <v>42369.818796296298</v>
+      </c>
+      <c r="K87" s="73">
+        <v>11.13</v>
+      </c>
+      <c r="L87" s="73">
+        <v>10.275</v>
+      </c>
+      <c r="M87" s="71">
+        <v>19.78</v>
+      </c>
+    </row>
+    <row r="88" spans="1:14">
+      <c r="A88" s="59">
+        <v>1</v>
+      </c>
+      <c r="B88" s="59">
+        <v>10</v>
+      </c>
+      <c r="C88" s="59">
+        <v>15</v>
+      </c>
+      <c r="D88" s="59">
+        <v>0</v>
+      </c>
+      <c r="E88" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F88" s="75">
+        <v>679.64</v>
+      </c>
+      <c r="J88" s="68">
+        <v>36841</v>
+      </c>
+      <c r="K88" s="73">
+        <v>22.992000000000001</v>
+      </c>
+      <c r="L88" s="73">
+        <v>22.9920399034783</v>
+      </c>
+      <c r="N88" s="59" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="89" spans="1:14">
+      <c r="A89" s="59">
+        <v>1</v>
+      </c>
+      <c r="B89" s="59">
+        <v>10</v>
+      </c>
+      <c r="C89" s="59">
+        <v>23</v>
+      </c>
+      <c r="D89" s="59">
+        <v>1</v>
+      </c>
+      <c r="E89" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Venda</v>
+      </c>
+      <c r="F89" s="75">
+        <v>679.64</v>
+      </c>
+      <c r="H89" s="59">
+        <v>11</v>
+      </c>
+      <c r="J89" s="68">
+        <v>41383</v>
+      </c>
+      <c r="K89" s="73">
+        <v>22.992000000000001</v>
+      </c>
+      <c r="L89" s="73">
+        <v>8.1098375610617399</v>
+      </c>
+      <c r="N89" s="59" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="90" spans="1:14">
+      <c r="A90" s="59">
+        <v>1</v>
+      </c>
+      <c r="B90" s="59">
+        <v>11</v>
+      </c>
+      <c r="C90" s="59">
+        <v>16</v>
+      </c>
+      <c r="D90" s="59">
+        <v>0</v>
+      </c>
+      <c r="E90" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F90" s="75">
+        <v>547.645126</v>
+      </c>
+      <c r="J90" s="68">
+        <v>41166</v>
+      </c>
+      <c r="K90" s="73">
+        <v>18.260000000000002</v>
+      </c>
+      <c r="L90" s="73">
+        <v>18.259999998612201</v>
+      </c>
+      <c r="N90" s="59" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="91" spans="1:14">
+      <c r="A91" s="59">
+        <v>1</v>
+      </c>
+      <c r="B91" s="59">
+        <v>11</v>
+      </c>
+      <c r="C91" s="59">
+        <v>17</v>
+      </c>
+      <c r="D91" s="59">
+        <v>0</v>
+      </c>
+      <c r="E91" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F91" s="75">
+        <v>1010.611</v>
+      </c>
+      <c r="J91" s="68">
+        <v>41377</v>
+      </c>
+      <c r="K91" s="73">
+        <v>19.79</v>
+      </c>
+      <c r="L91" s="73">
+        <v>19.7899983277443</v>
+      </c>
+    </row>
+    <row r="92" spans="1:14">
+      <c r="A92" s="59">
+        <v>1</v>
+      </c>
+      <c r="B92" s="59">
+        <v>11</v>
+      </c>
+      <c r="C92" s="59">
+        <v>24</v>
+      </c>
+      <c r="D92" s="59">
+        <v>0</v>
+      </c>
+      <c r="E92" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F92" s="75">
+        <v>280.07</v>
+      </c>
+      <c r="H92" s="59">
+        <v>10</v>
+      </c>
+      <c r="I92" s="59">
+        <v>23</v>
+      </c>
+      <c r="J92" s="68">
+        <v>41383.000011574077</v>
+      </c>
+      <c r="K92" s="73">
+        <v>55.794199999999996</v>
+      </c>
+      <c r="L92" s="73">
+        <v>19.6799728639268</v>
+      </c>
+      <c r="N92" s="59" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="93" spans="1:14">
+      <c r="A93" s="59">
+        <v>1</v>
+      </c>
+      <c r="B93" s="59">
+        <v>11</v>
+      </c>
+      <c r="C93" s="59">
+        <v>25</v>
+      </c>
+      <c r="D93" s="59">
+        <v>1</v>
+      </c>
+      <c r="E93" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Venda</v>
+      </c>
+      <c r="F93" s="75">
+        <v>1838.3261259999999</v>
+      </c>
+      <c r="H93" s="59">
+        <v>5</v>
+      </c>
+      <c r="J93" s="68">
+        <v>41439</v>
+      </c>
+      <c r="K93" s="73">
+        <v>24.819500000000001</v>
+      </c>
+      <c r="L93" s="73">
+        <v>18.949999952293499</v>
+      </c>
+      <c r="N93" s="59" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="94" spans="1:14">
+      <c r="A94" s="59">
+        <v>1</v>
+      </c>
+      <c r="B94" s="59">
+        <v>12</v>
+      </c>
+      <c r="C94" s="59">
+        <v>32</v>
+      </c>
+      <c r="D94" s="59">
+        <v>0</v>
+      </c>
+      <c r="E94" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F94" s="75">
+        <v>5006.5078999999996</v>
+      </c>
+      <c r="J94" s="68">
+        <v>41166.000011574077</v>
+      </c>
+      <c r="K94" s="73">
+        <v>1.9974000000000001</v>
+      </c>
+      <c r="L94" s="73">
+        <v>1.9974000000000001</v>
+      </c>
+      <c r="N94" s="59" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="95" spans="1:14">
+      <c r="A95" s="59">
+        <v>1</v>
+      </c>
+      <c r="B95" s="59">
+        <v>12</v>
+      </c>
+      <c r="C95" s="59">
+        <v>33</v>
+      </c>
+      <c r="D95" s="59">
+        <v>1</v>
+      </c>
+      <c r="E95" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Venda</v>
+      </c>
+      <c r="F95" s="75">
+        <v>5006.5078999999996</v>
+      </c>
+      <c r="H95" s="59">
+        <v>13</v>
+      </c>
+      <c r="J95" s="68">
+        <v>41385</v>
+      </c>
+      <c r="K95" s="73">
+        <v>1.9974000000000001</v>
+      </c>
+      <c r="L95" s="73">
+        <v>2.0725623942389002</v>
+      </c>
+      <c r="N95" s="59" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="96" spans="1:14">
+      <c r="A96" s="59">
+        <v>1</v>
+      </c>
+      <c r="B96" s="59">
+        <v>13</v>
+      </c>
+      <c r="C96" s="59">
+        <v>34</v>
+      </c>
+      <c r="D96" s="59">
+        <v>0</v>
+      </c>
+      <c r="E96" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F96" s="75">
+        <v>394.85</v>
+      </c>
+      <c r="H96" s="59">
+        <v>12</v>
+      </c>
+      <c r="I96" s="59">
+        <v>33</v>
+      </c>
+      <c r="J96" s="68">
+        <v>41385.000011574077</v>
+      </c>
+      <c r="K96" s="73">
+        <v>25.3261</v>
+      </c>
+      <c r="L96" s="73">
+        <v>26.279093326579702</v>
+      </c>
+      <c r="N96" s="59" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="97" spans="1:14">
+      <c r="A97" s="59">
+        <v>1</v>
+      </c>
+      <c r="B97" s="59">
+        <v>13</v>
+      </c>
+      <c r="C97" s="59">
+        <v>42</v>
+      </c>
+      <c r="D97" s="59">
+        <v>1</v>
+      </c>
+      <c r="E97" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Venda</v>
+      </c>
+      <c r="F97" s="75">
+        <v>394.85</v>
+      </c>
+      <c r="J97" s="68">
+        <v>41436.000011574077</v>
+      </c>
+      <c r="K97" s="73">
+        <v>25.3261</v>
+      </c>
+      <c r="L97" s="73">
+        <v>24.609000886412499</v>
+      </c>
+      <c r="N97" s="59" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="98" spans="1:14">
+      <c r="A98" s="59">
+        <v>1</v>
+      </c>
+      <c r="B98" s="59">
+        <v>14</v>
+      </c>
+      <c r="C98" s="59">
+        <v>35</v>
+      </c>
+      <c r="D98" s="59">
+        <v>0</v>
+      </c>
+      <c r="E98" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F98" s="75">
+        <v>21.84</v>
+      </c>
+      <c r="J98" s="68">
+        <v>41201</v>
+      </c>
+      <c r="K98" s="73">
+        <v>549.56460000000004</v>
+      </c>
+      <c r="L98" s="73">
+        <v>549.56456043955995</v>
+      </c>
+      <c r="N98" s="59" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="99" spans="1:14">
+      <c r="A99" s="59">
+        <v>1</v>
+      </c>
+      <c r="B99" s="59">
+        <v>14</v>
+      </c>
+      <c r="C99" s="59">
+        <v>36</v>
+      </c>
+      <c r="D99" s="59">
+        <v>1</v>
+      </c>
+      <c r="E99" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Venda</v>
+      </c>
+      <c r="F99" s="75">
+        <v>21.84</v>
+      </c>
+      <c r="J99" s="68">
+        <v>41436</v>
+      </c>
+      <c r="K99" s="73">
+        <v>549.56460000000004</v>
+      </c>
+      <c r="L99" s="73">
+        <v>547.44001831501805</v>
+      </c>
+      <c r="N99" s="59" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="100" spans="1:14">
+      <c r="A100" s="59">
+        <v>1</v>
+      </c>
+      <c r="B100" s="59">
+        <v>15</v>
+      </c>
+      <c r="C100" s="59">
+        <v>98</v>
+      </c>
+      <c r="D100" s="59">
+        <v>0</v>
+      </c>
+      <c r="E100" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F100" s="75">
+        <v>112.246</v>
+      </c>
+      <c r="J100" s="68">
+        <v>42219.795451388891</v>
+      </c>
+      <c r="K100" s="73">
+        <v>8.9090000000000007</v>
+      </c>
+      <c r="L100" s="73">
+        <v>8.9090034388753203</v>
+      </c>
+    </row>
+    <row r="101" spans="1:14">
+      <c r="A101" s="59">
+        <v>1</v>
+      </c>
+      <c r="B101" s="59">
+        <v>15</v>
+      </c>
+      <c r="C101" s="59">
+        <v>122</v>
+      </c>
+      <c r="D101" s="59">
+        <v>0</v>
+      </c>
+      <c r="E101" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F101" s="75">
+        <v>5585.1589999999997</v>
+      </c>
+      <c r="J101" s="68">
+        <v>42635.715057870373</v>
+      </c>
+      <c r="K101" s="73">
+        <v>8.952</v>
+      </c>
+      <c r="L101" s="73">
+        <v>8.952</v>
+      </c>
+      <c r="M101" s="71">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102" spans="1:14">
+      <c r="A102" s="59">
+        <v>1</v>
+      </c>
+      <c r="B102" s="59">
+        <v>16</v>
+      </c>
+      <c r="C102" s="59">
+        <v>101</v>
+      </c>
+      <c r="D102" s="59">
+        <v>0</v>
+      </c>
+      <c r="E102" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F102" s="75">
+        <v>160.75280000000001</v>
+      </c>
+      <c r="H102" s="59">
+        <v>1</v>
+      </c>
+      <c r="I102" s="59">
+        <v>100</v>
+      </c>
+      <c r="J102" s="68">
+        <v>42279.463807870372</v>
+      </c>
+      <c r="K102" s="73">
+        <v>280.20139999999998</v>
+      </c>
+      <c r="L102" s="73">
+        <v>323.52997894904399</v>
+      </c>
+      <c r="N102" s="59" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="103" spans="1:14">
+      <c r="A103" s="59">
+        <v>1</v>
+      </c>
+      <c r="B103" s="59">
+        <v>17</v>
+      </c>
+      <c r="C103" s="59">
+        <v>105</v>
+      </c>
+      <c r="D103" s="59">
+        <v>0</v>
+      </c>
+      <c r="E103" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F103" s="75">
+        <v>15</v>
+      </c>
+      <c r="J103" s="68">
+        <v>42325.618148148147</v>
+      </c>
+      <c r="K103" s="73">
+        <v>63.64</v>
+      </c>
+      <c r="L103" s="73">
+        <v>63.64</v>
+      </c>
+      <c r="M103" s="71">
+        <v>14.95</v>
+      </c>
+    </row>
+    <row r="104" spans="1:14">
+      <c r="A104" s="59">
+        <v>1</v>
+      </c>
+      <c r="B104" s="59">
+        <v>17</v>
+      </c>
+      <c r="C104" s="59">
+        <v>125</v>
+      </c>
+      <c r="D104" s="59">
+        <v>1</v>
+      </c>
+      <c r="E104" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Venda</v>
+      </c>
+      <c r="F104" s="75">
+        <v>15</v>
+      </c>
+      <c r="J104" s="68">
+        <v>42731.461006944446</v>
+      </c>
+      <c r="K104" s="73">
+        <v>63.64</v>
+      </c>
+      <c r="L104" s="73">
+        <v>40.207000000000001</v>
+      </c>
+      <c r="M104" s="71">
+        <v>14.95</v>
+      </c>
+    </row>
+    <row r="105" spans="1:14">
+      <c r="A105" s="59">
+        <v>1</v>
+      </c>
+      <c r="B105" s="59">
+        <v>18</v>
+      </c>
+      <c r="C105" s="59">
+        <v>109</v>
+      </c>
+      <c r="D105" s="59">
+        <v>0</v>
+      </c>
+      <c r="E105" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F105" s="75">
+        <v>235</v>
+      </c>
+      <c r="J105" s="68">
+        <v>42394.669849537036</v>
+      </c>
+      <c r="K105" s="73">
+        <v>170</v>
+      </c>
+      <c r="L105" s="73">
+        <v>170</v>
+      </c>
+      <c r="M105" s="71">
+        <v>79.900000000000006</v>
+      </c>
+    </row>
+    <row r="106" spans="1:14">
+      <c r="A106" s="59">
+        <v>1</v>
+      </c>
+      <c r="B106" s="59">
+        <v>18</v>
+      </c>
+      <c r="C106" s="59">
+        <v>110</v>
+      </c>
+      <c r="D106" s="59">
+        <v>0</v>
+      </c>
+      <c r="E106" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F106" s="75">
+        <v>55</v>
+      </c>
+      <c r="J106" s="68">
+        <v>42394.669861111113</v>
+      </c>
+      <c r="K106" s="73">
+        <v>169.97</v>
+      </c>
+      <c r="L106" s="73">
+        <v>169.97</v>
+      </c>
+      <c r="M106" s="71">
+        <v>14.95</v>
+      </c>
+    </row>
+    <row r="107" spans="1:14">
+      <c r="A107" s="59">
+        <v>1</v>
+      </c>
+      <c r="B107" s="59">
+        <v>18</v>
+      </c>
+      <c r="C107" s="59">
+        <v>111</v>
+      </c>
+      <c r="D107" s="59">
+        <v>1</v>
+      </c>
+      <c r="E107" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Venda</v>
+      </c>
+      <c r="F107" s="75">
+        <v>290</v>
+      </c>
+      <c r="J107" s="68">
+        <v>42544.806469907409</v>
+      </c>
+      <c r="K107" s="73">
+        <v>169.99430000000001</v>
+      </c>
+      <c r="L107" s="73">
+        <v>181.5</v>
+      </c>
+      <c r="M107" s="71">
+        <v>105.27</v>
+      </c>
+    </row>
+    <row r="108" spans="1:14">
+      <c r="A108" s="59">
+        <v>1</v>
+      </c>
+      <c r="B108" s="59">
+        <v>19</v>
+      </c>
+      <c r="C108" s="59">
+        <v>108</v>
+      </c>
+      <c r="D108" s="59">
+        <v>0</v>
+      </c>
+      <c r="E108" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F108" s="75">
+        <v>0.53749999999999998</v>
+      </c>
+      <c r="J108" s="68">
+        <v>42387.492534722223</v>
+      </c>
+      <c r="K108" s="73">
+        <v>1860.4650999999999</v>
+      </c>
+      <c r="L108" s="73">
+        <v>1860.4651162790699</v>
+      </c>
+    </row>
+    <row r="109" spans="1:14">
+      <c r="A109" s="59">
+        <v>1</v>
+      </c>
+      <c r="B109" s="59">
+        <v>23</v>
+      </c>
+      <c r="C109" s="59">
+        <v>123</v>
+      </c>
+      <c r="D109" s="59">
+        <v>0</v>
+      </c>
+      <c r="E109" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F109" s="75">
+        <v>175</v>
+      </c>
+      <c r="J109" s="68">
+        <v>42642.772696759261</v>
+      </c>
+      <c r="K109" s="73">
+        <v>33.215000000000003</v>
+      </c>
+      <c r="L109" s="73">
+        <v>33.215000000000003</v>
+      </c>
+      <c r="M109" s="71">
+        <v>12.41</v>
+      </c>
+    </row>
+    <row r="110" spans="1:14">
+      <c r="A110" s="59">
+        <v>1</v>
+      </c>
+      <c r="B110" s="59">
+        <v>23</v>
+      </c>
+      <c r="C110" s="59">
+        <v>131</v>
+      </c>
+      <c r="D110" s="59">
+        <v>0</v>
+      </c>
+      <c r="E110" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F110" s="75">
+        <v>200</v>
+      </c>
+      <c r="J110" s="68">
+        <v>42752.496111111112</v>
+      </c>
+      <c r="K110" s="73">
+        <v>31.45</v>
+      </c>
+      <c r="L110" s="73">
+        <v>31.45</v>
+      </c>
+      <c r="M110" s="71">
+        <v>14.57</v>
+      </c>
+    </row>
+    <row r="111" spans="1:14">
+      <c r="A111" s="59">
+        <v>1</v>
+      </c>
+      <c r="B111" s="59">
+        <v>23</v>
+      </c>
+      <c r="C111" s="59">
+        <v>134</v>
+      </c>
+      <c r="D111" s="59">
+        <v>2</v>
+      </c>
+      <c r="E111" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Venda</v>
+      </c>
+      <c r="F111" s="75">
+        <v>0</v>
+      </c>
+      <c r="J111" s="68">
+        <v>42676.715624999997</v>
+      </c>
+      <c r="L111" s="73">
+        <v>52.5</v>
+      </c>
+      <c r="M111" s="71">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112" spans="1:14">
+      <c r="A112" s="59">
+        <v>1</v>
+      </c>
+      <c r="B112" s="59">
+        <v>23</v>
+      </c>
+      <c r="C112" s="59">
+        <v>140</v>
+      </c>
+      <c r="D112" s="59">
+        <v>1</v>
+      </c>
+      <c r="E112" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Venda</v>
+      </c>
+      <c r="F112" s="75">
+        <v>375</v>
+      </c>
+      <c r="J112" s="68">
+        <v>42835.43141203704</v>
+      </c>
+      <c r="K112" s="73">
+        <v>32.273699999999998</v>
+      </c>
+      <c r="L112" s="73">
+        <v>33.799999999999997</v>
+      </c>
+      <c r="M112" s="71">
+        <v>15.34</v>
+      </c>
+    </row>
+    <row r="113" spans="1:14">
+      <c r="A113" s="59">
+        <v>1</v>
+      </c>
+      <c r="B113" s="59">
+        <v>24</v>
+      </c>
+      <c r="C113" s="59">
+        <v>137</v>
+      </c>
+      <c r="D113" s="59">
+        <v>0</v>
+      </c>
+      <c r="E113" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F113" s="75">
+        <v>25</v>
+      </c>
+      <c r="J113" s="68">
+        <v>42814.418206018519</v>
+      </c>
+      <c r="K113" s="73">
+        <v>37.17</v>
+      </c>
+      <c r="L113" s="73">
+        <v>37.17</v>
+      </c>
+      <c r="M113" s="71">
+        <v>14.95</v>
+      </c>
+    </row>
+    <row r="114" spans="1:14">
+      <c r="A114" s="59">
+        <v>1</v>
+      </c>
+      <c r="B114" s="59">
+        <v>24</v>
+      </c>
+      <c r="C114" s="59">
+        <v>145</v>
+      </c>
+      <c r="D114" s="59">
+        <v>1</v>
+      </c>
+      <c r="E114" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Venda</v>
+      </c>
+      <c r="F114" s="75">
+        <v>25</v>
+      </c>
+      <c r="J114" s="68">
+        <v>42881.460057870368</v>
+      </c>
+      <c r="K114" s="73">
+        <v>37.17</v>
+      </c>
+      <c r="L114" s="73">
+        <v>37.202488000000002</v>
+      </c>
+      <c r="M114" s="71">
+        <v>14.98</v>
+      </c>
+    </row>
+    <row r="115" spans="1:14">
+      <c r="A115" s="59">
+        <v>1</v>
+      </c>
+      <c r="B115" s="59">
+        <v>25</v>
+      </c>
+      <c r="C115" s="59">
+        <v>136</v>
+      </c>
+      <c r="D115" s="59">
+        <v>0</v>
+      </c>
+      <c r="E115" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F115" s="75">
+        <v>5</v>
+      </c>
+      <c r="J115" s="68">
+        <v>42814.417696759258</v>
+      </c>
+      <c r="K115" s="73">
+        <v>204.52</v>
+      </c>
+      <c r="L115" s="73">
+        <v>204.52</v>
+      </c>
+      <c r="M115" s="71">
+        <v>14.95</v>
+      </c>
+    </row>
+    <row r="116" spans="1:14">
+      <c r="A116" s="59">
+        <v>1</v>
+      </c>
+      <c r="B116" s="59">
+        <v>25</v>
+      </c>
+      <c r="C116" s="59">
+        <v>146</v>
+      </c>
+      <c r="D116" s="59">
+        <v>1</v>
+      </c>
+      <c r="E116" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Venda</v>
+      </c>
+      <c r="F116" s="75">
+        <v>5</v>
+      </c>
+      <c r="J116" s="68">
+        <v>42881.463125000002</v>
+      </c>
+      <c r="K116" s="73">
+        <v>204.52</v>
+      </c>
+      <c r="L116" s="73">
+        <v>198.079802</v>
+      </c>
+      <c r="M116" s="71">
+        <v>14.98</v>
+      </c>
+    </row>
+    <row r="117" spans="1:14">
+      <c r="J117" s="68"/>
+    </row>
+    <row r="118" spans="1:14">
+      <c r="J118" s="68"/>
+    </row>
+    <row r="119" spans="1:14">
+      <c r="A119" s="59">
+        <v>2</v>
+      </c>
+      <c r="B119" s="59">
+        <v>7</v>
+      </c>
+      <c r="C119" s="59">
+        <v>139</v>
+      </c>
+      <c r="D119" s="59">
+        <v>5</v>
+      </c>
+      <c r="E119" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Venda</v>
+      </c>
+      <c r="F119" s="75">
+        <v>6225</v>
+      </c>
+      <c r="J119" s="68">
+        <v>42822.45480324074</v>
+      </c>
+      <c r="K119" s="73">
+        <v>7.5839999999999996</v>
+      </c>
+      <c r="L119" s="73">
+        <v>7.5839999999999996</v>
+      </c>
+      <c r="M119" s="71">
+        <v>33.31</v>
+      </c>
+      <c r="N119" s="59" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="120" spans="1:14">
+      <c r="A120" s="59">
+        <v>2</v>
+      </c>
+      <c r="B120" s="59">
+        <v>7</v>
+      </c>
+      <c r="C120" s="59">
+        <v>142</v>
+      </c>
+      <c r="D120" s="59">
+        <v>5</v>
+      </c>
+      <c r="E120" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Venda</v>
+      </c>
+      <c r="F120" s="75">
+        <v>1671</v>
+      </c>
+      <c r="J120" s="68">
+        <v>42871.778969907406</v>
+      </c>
+      <c r="K120" s="73">
+        <v>6.7969999999999997</v>
+      </c>
+      <c r="L120" s="73">
+        <v>6.7969999999999997</v>
+      </c>
+      <c r="M120" s="71">
+        <v>15.07</v>
+      </c>
+      <c r="N120" s="59" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="121" spans="1:14">
+      <c r="A121" s="59">
+        <v>2</v>
+      </c>
+      <c r="B121" s="59">
+        <v>7</v>
+      </c>
+      <c r="C121" s="59">
+        <v>144</v>
+      </c>
+      <c r="D121" s="59">
+        <v>5</v>
+      </c>
+      <c r="E121" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Venda</v>
+      </c>
+      <c r="F121" s="75">
+        <v>2001</v>
+      </c>
+      <c r="J121" s="68">
+        <v>42871.788263888891</v>
+      </c>
+      <c r="K121" s="73">
+        <v>6.7960000000000003</v>
+      </c>
+      <c r="L121" s="73">
+        <v>6.7960000000000003</v>
+      </c>
+      <c r="M121" s="71">
+        <v>15.34</v>
+      </c>
+      <c r="N121" s="59" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="122" spans="1:14">
+      <c r="A122" s="59">
+        <v>2</v>
+      </c>
+      <c r="B122" s="59">
+        <v>7</v>
+      </c>
+      <c r="C122" s="59">
+        <v>155</v>
+      </c>
+      <c r="D122" s="59">
+        <v>0</v>
+      </c>
+      <c r="E122" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F122" s="75">
+        <v>2075</v>
+      </c>
+      <c r="J122" s="68">
+        <v>42822.454814814817</v>
+      </c>
+      <c r="K122" s="73">
+        <v>22.751999999999999</v>
+      </c>
+      <c r="L122" s="73">
+        <v>22.751999999999999</v>
+      </c>
+      <c r="M122" s="71">
+        <v>33.31</v>
+      </c>
+      <c r="N122" s="59" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="123" spans="1:14">
+      <c r="A123" s="59">
+        <v>2</v>
+      </c>
+      <c r="B123" s="59">
+        <v>7</v>
+      </c>
+      <c r="C123" s="59">
+        <v>156</v>
+      </c>
+      <c r="D123" s="59">
+        <v>0</v>
+      </c>
+      <c r="E123" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F123" s="75">
+        <v>557</v>
+      </c>
+      <c r="J123" s="68">
+        <v>42871.778981481482</v>
+      </c>
+      <c r="K123" s="73">
+        <v>20.390999999999998</v>
+      </c>
+      <c r="L123" s="73">
+        <v>20.390999999999998</v>
+      </c>
+      <c r="M123" s="71">
+        <v>15.07</v>
+      </c>
+      <c r="N123" s="59" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="124" spans="1:14">
+      <c r="A124" s="59">
+        <v>2</v>
+      </c>
+      <c r="B124" s="59">
+        <v>7</v>
+      </c>
+      <c r="C124" s="59">
+        <v>157</v>
+      </c>
+      <c r="D124" s="59">
+        <v>0</v>
+      </c>
+      <c r="E124" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F124" s="75">
+        <v>667</v>
+      </c>
+      <c r="J124" s="68">
+        <v>42871.788275462961</v>
+      </c>
+      <c r="K124" s="73">
+        <v>20.388000000000002</v>
+      </c>
+      <c r="L124" s="73">
+        <v>20.388000000000002</v>
+      </c>
+      <c r="M124" s="71">
+        <v>15.34</v>
+      </c>
+      <c r="N124" s="59" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="125" spans="1:14">
+      <c r="A125" s="59">
+        <v>2</v>
+      </c>
+      <c r="B125" s="59">
+        <v>7</v>
+      </c>
+      <c r="C125" s="59">
+        <v>162</v>
+      </c>
+      <c r="D125" s="59">
+        <v>1</v>
+      </c>
+      <c r="E125" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Venda</v>
+      </c>
+      <c r="F125" s="75">
+        <v>2642</v>
+      </c>
+      <c r="J125" s="68">
+        <v>43069.39916666667</v>
+      </c>
+      <c r="K125" s="73">
+        <v>22.2453</v>
+      </c>
+      <c r="L125" s="73">
+        <v>25.99</v>
+      </c>
+      <c r="M125" s="71">
+        <v>59.61</v>
+      </c>
+    </row>
+    <row r="126" spans="1:14">
+      <c r="A126" s="59">
+        <v>2</v>
+      </c>
+      <c r="B126" s="59">
+        <v>7</v>
+      </c>
+      <c r="C126" s="59">
+        <v>163</v>
+      </c>
+      <c r="D126" s="59">
+        <v>1</v>
+      </c>
+      <c r="E126" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Venda</v>
+      </c>
+      <c r="F126" s="75">
+        <v>657</v>
+      </c>
+      <c r="J126" s="68">
+        <v>43069.400335648148</v>
+      </c>
+      <c r="K126" s="73">
+        <v>20.388000000000002</v>
+      </c>
+      <c r="L126" s="73">
+        <v>25.984999999999999</v>
+      </c>
+      <c r="M126" s="71">
+        <v>15.76</v>
+      </c>
+    </row>
+    <row r="127" spans="1:14">
+      <c r="A127" s="59">
+        <v>2</v>
+      </c>
+      <c r="B127" s="59">
+        <v>15</v>
+      </c>
+      <c r="C127" s="59">
+        <v>124</v>
+      </c>
+      <c r="D127" s="59">
+        <v>0</v>
+      </c>
+      <c r="E127" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F127" s="75">
+        <v>2607.6527000000001</v>
+      </c>
+      <c r="J127" s="68">
+        <v>42696.26803240741</v>
+      </c>
+      <c r="K127" s="73">
+        <v>8.82</v>
+      </c>
+      <c r="L127" s="73">
+        <v>8.82</v>
+      </c>
+      <c r="M127" s="71">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128" spans="1:14">
+      <c r="A128" s="59">
+        <v>2</v>
+      </c>
+      <c r="B128" s="59">
+        <v>15</v>
+      </c>
+      <c r="C128" s="59">
+        <v>160</v>
+      </c>
+      <c r="D128" s="59">
+        <v>1</v>
+      </c>
+      <c r="E128" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Venda</v>
+      </c>
+      <c r="F128" s="75">
+        <v>2500</v>
+      </c>
+      <c r="H128" s="59">
+        <v>16</v>
+      </c>
+      <c r="J128" s="68">
+        <v>43045.551990740743</v>
+      </c>
+      <c r="K128" s="73">
+        <v>8.82</v>
+      </c>
+      <c r="L128" s="73">
+        <v>10.080055</v>
+      </c>
+    </row>
+    <row r="129" spans="1:14">
+      <c r="A129" s="59">
+        <v>2</v>
+      </c>
+      <c r="B129" s="59">
+        <v>15</v>
+      </c>
+      <c r="C129" s="59">
+        <v>164</v>
+      </c>
+      <c r="D129" s="59">
+        <v>0</v>
+      </c>
+      <c r="E129" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F129" s="75">
+        <v>2918.857</v>
+      </c>
+      <c r="J129" s="68">
+        <v>43109.468252314815</v>
+      </c>
+      <c r="K129" s="73">
+        <v>10.2369</v>
+      </c>
+      <c r="L129" s="73">
+        <v>10.236924999999999</v>
+      </c>
+      <c r="M129" s="71">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130" spans="1:14">
+      <c r="A130" s="59">
+        <v>2</v>
+      </c>
+      <c r="B130" s="59">
+        <v>16</v>
+      </c>
+      <c r="C130" s="59">
+        <v>161</v>
+      </c>
+      <c r="D130" s="59">
+        <v>0</v>
+      </c>
+      <c r="E130" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F130" s="75">
+        <v>57.306899999999999</v>
+      </c>
+      <c r="I130" s="59">
+        <v>160</v>
+      </c>
+      <c r="J130" s="68">
+        <v>43046.552071759259</v>
+      </c>
+      <c r="K130" s="73">
+        <v>384.7704</v>
+      </c>
+      <c r="L130" s="73">
+        <v>439.74</v>
+      </c>
+    </row>
+    <row r="131" spans="1:14">
+      <c r="A131" s="59">
+        <v>2</v>
+      </c>
+      <c r="B131" s="59">
+        <v>22</v>
+      </c>
+      <c r="C131" s="59">
+        <v>112</v>
+      </c>
+      <c r="D131" s="59">
+        <v>0</v>
+      </c>
+      <c r="E131" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F131" s="75">
+        <v>15925</v>
+      </c>
+      <c r="J131" s="68">
+        <v>42328.817766203705</v>
+      </c>
+      <c r="K131" s="73">
+        <v>1.939684873</v>
+      </c>
+      <c r="L131" s="73">
+        <v>1.939684873</v>
+      </c>
+    </row>
+    <row r="132" spans="1:14">
+      <c r="A132" s="59">
+        <v>2</v>
+      </c>
+      <c r="B132" s="59">
+        <v>22</v>
+      </c>
+      <c r="C132" s="59">
+        <v>113</v>
+      </c>
+      <c r="D132" s="59">
+        <v>0</v>
+      </c>
+      <c r="E132" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F132" s="75">
+        <v>191</v>
+      </c>
+      <c r="J132" s="68">
+        <v>42474.688692129632</v>
+      </c>
+      <c r="K132" s="73">
+        <v>0</v>
+      </c>
+      <c r="L132" s="73">
+        <v>0</v>
+      </c>
+      <c r="M132" s="71">
+        <v>0</v>
+      </c>
+      <c r="N132" s="59" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="133" spans="1:14">
+      <c r="A133" s="59">
+        <v>2</v>
+      </c>
+      <c r="B133" s="59">
+        <v>22</v>
+      </c>
+      <c r="C133" s="59">
+        <v>114</v>
+      </c>
+      <c r="D133" s="59">
+        <v>0</v>
+      </c>
+      <c r="E133" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Compra</v>
+      </c>
+      <c r="F133" s="75">
+        <v>468</v>
+      </c>
+      <c r="J133" s="68">
+        <v>42479.69158564815</v>
+      </c>
+      <c r="K133" s="73">
+        <v>0</v>
+      </c>
+      <c r="L133" s="73">
+        <v>0</v>
+      </c>
+      <c r="M133" s="71">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134" spans="1:14">
+      <c r="A134" s="59">
+        <v>2</v>
+      </c>
+      <c r="B134" s="59">
+        <v>22</v>
+      </c>
+      <c r="C134" s="59">
+        <v>115</v>
+      </c>
+      <c r="D134" s="59">
+        <v>1</v>
+      </c>
+      <c r="E134" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Venda</v>
+      </c>
+      <c r="F134" s="75">
+        <v>11484</v>
+      </c>
+      <c r="J134" s="68">
+        <v>42606.428784722222</v>
+      </c>
+      <c r="K134" s="73">
+        <v>1.9397</v>
+      </c>
+      <c r="L134" s="73">
+        <v>1.2090000000000001</v>
+      </c>
+      <c r="M134" s="71">
+        <v>15.27</v>
+      </c>
+    </row>
+    <row r="135" spans="1:14">
+      <c r="A135" s="59">
+        <v>2</v>
+      </c>
+      <c r="B135" s="59">
+        <v>22</v>
+      </c>
+      <c r="C135" s="59">
+        <v>116</v>
+      </c>
+      <c r="D135" s="59">
+        <v>2</v>
+      </c>
+      <c r="E135" s="59" t="str">
+        <f t="shared" si="2"/>
+        <v>Venda</v>
+      </c>
+      <c r="F135" s="75">
+        <v>0</v>
+      </c>
+      <c r="J135" s="68">
+        <v>42370.474548611113</v>
+      </c>
+      <c r="L135" s="73">
+        <v>0.64</v>
+      </c>
+      <c r="M135" s="71">
+        <v>0</v>
+      </c>
+      <c r="N135" s="59" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="136" spans="1:14">
+      <c r="A136" s="59">
+        <v>2</v>
+      </c>
+      <c r="B136" s="59">
+        <v>22</v>
+      </c>
+      <c r="C136" s="59">
+        <v>117</v>
+      </c>
+      <c r="D136" s="59">
+        <v>2</v>
+      </c>
+      <c r="E136" s="59" t="str">
+        <f t="shared" ref="E136:E145" si="3">IF(D136=0,"Compra","Venda")</f>
+        <v>Venda</v>
+      </c>
+      <c r="F136" s="75">
+        <v>0</v>
+      </c>
+      <c r="J136" s="68">
+        <v>42401.474733796298</v>
+      </c>
+      <c r="L136" s="73">
+        <v>0.32</v>
+      </c>
+      <c r="M136" s="71">
+        <v>0</v>
+      </c>
+      <c r="N136" s="59" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="137" spans="1:14">
+      <c r="A137" s="59">
+        <v>2</v>
+      </c>
+      <c r="B137" s="59">
+        <v>22</v>
+      </c>
+      <c r="C137" s="59">
+        <v>118</v>
+      </c>
+      <c r="D137" s="59">
+        <v>2</v>
+      </c>
+      <c r="E137" s="59" t="str">
+        <f t="shared" si="3"/>
+        <v>Venda</v>
+      </c>
+      <c r="F137" s="75">
+        <v>0</v>
+      </c>
+      <c r="J137" s="68">
+        <v>42461.474942129629</v>
+      </c>
+      <c r="L137" s="73">
+        <v>12.29</v>
+      </c>
+      <c r="M137" s="71">
+        <v>0</v>
+      </c>
+      <c r="N137" s="59" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="138" spans="1:14">
+      <c r="A138" s="59">
+        <v>2</v>
+      </c>
+      <c r="B138" s="59">
+        <v>22</v>
+      </c>
+      <c r="C138" s="59">
+        <v>119</v>
+      </c>
+      <c r="D138" s="59">
+        <v>2</v>
+      </c>
+      <c r="E138" s="59" t="str">
+        <f t="shared" si="3"/>
+        <v>Venda</v>
+      </c>
+      <c r="F138" s="75">
+        <v>0</v>
+      </c>
+      <c r="J138" s="68">
+        <v>42491.47515046296</v>
+      </c>
+      <c r="L138" s="73">
+        <v>18.7</v>
+      </c>
+      <c r="M138" s="71">
+        <v>0</v>
+      </c>
+      <c r="N138" s="59" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="139" spans="1:14">
+      <c r="A139" s="59">
+        <v>2</v>
+      </c>
+      <c r="B139" s="59">
+        <v>22</v>
+      </c>
+      <c r="C139" s="59">
+        <v>120</v>
+      </c>
+      <c r="D139" s="59">
+        <v>2</v>
+      </c>
+      <c r="E139" s="59" t="str">
+        <f t="shared" si="3"/>
+        <v>Venda</v>
+      </c>
+      <c r="F139" s="75">
+        <v>0</v>
+      </c>
+      <c r="J139" s="68">
+        <v>42522.475381944445</v>
+      </c>
+      <c r="L139" s="73">
+        <v>10.94</v>
+      </c>
+      <c r="M139" s="71">
+        <v>0</v>
+      </c>
+      <c r="N139" s="59" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="140" spans="1:14">
+      <c r="A140" s="59">
+        <v>2</v>
+      </c>
+      <c r="B140" s="59">
+        <v>22</v>
+      </c>
+      <c r="C140" s="59">
+        <v>121</v>
+      </c>
+      <c r="D140" s="59">
+        <v>2</v>
+      </c>
+      <c r="E140" s="59" t="str">
+        <f t="shared" si="3"/>
+        <v>Venda</v>
+      </c>
+      <c r="F140" s="75">
+        <v>0</v>
+      </c>
+      <c r="J140" s="68">
+        <v>42552.475578703707</v>
+      </c>
+      <c r="L140" s="73">
+        <v>1.4</v>
+      </c>
+      <c r="M140" s="71">
+        <v>0</v>
+      </c>
+      <c r="N140" s="59" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="141" spans="1:14">
+      <c r="A141" s="59">
+        <v>2</v>
+      </c>
+      <c r="B141" s="59">
+        <v>22</v>
+      </c>
+      <c r="C141" s="59">
+        <v>132</v>
+      </c>
+      <c r="D141" s="59">
+        <v>1</v>
+      </c>
+      <c r="E141" s="59" t="str">
+        <f t="shared" si="3"/>
+        <v>Venda</v>
+      </c>
+      <c r="F141" s="75">
+        <v>5100</v>
+      </c>
+      <c r="J141" s="68">
+        <v>42711.564363425925</v>
+      </c>
+      <c r="K141" s="73">
+        <v>1.6890000000000001</v>
+      </c>
+      <c r="L141" s="73">
+        <v>1.3049999999999999</v>
+      </c>
+      <c r="M141" s="71">
+        <v>14.62</v>
+      </c>
+    </row>
+    <row r="142" spans="1:14">
+      <c r="A142" s="59">
+        <v>2</v>
+      </c>
+      <c r="B142" s="59">
+        <v>23</v>
+      </c>
+      <c r="C142" s="59">
+        <v>133</v>
+      </c>
+      <c r="D142" s="59">
+        <v>0</v>
+      </c>
+      <c r="E142" s="59" t="str">
+        <f t="shared" si="3"/>
+        <v>Compra</v>
+      </c>
+      <c r="F142" s="75">
+        <v>470</v>
+      </c>
+      <c r="J142" s="68">
+        <v>42740.566516203704</v>
+      </c>
+      <c r="K142" s="73">
+        <v>31.8</v>
+      </c>
+      <c r="L142" s="73">
+        <v>31.8</v>
+      </c>
+      <c r="M142" s="71">
+        <v>15.5</v>
+      </c>
+    </row>
+    <row r="143" spans="1:14">
+      <c r="A143" s="59">
+        <v>2</v>
+      </c>
+      <c r="B143" s="59">
+        <v>23</v>
+      </c>
+      <c r="C143" s="59">
+        <v>141</v>
+      </c>
+      <c r="D143" s="59">
+        <v>1</v>
+      </c>
+      <c r="E143" s="59" t="str">
+        <f t="shared" si="3"/>
+        <v>Venda</v>
+      </c>
+      <c r="F143" s="75">
+        <v>470</v>
+      </c>
+      <c r="J143" s="68">
+        <v>42835.433761574073</v>
+      </c>
+      <c r="K143" s="73">
+        <v>31.6511</v>
+      </c>
+      <c r="L143" s="73">
+        <v>33.799999999999997</v>
+      </c>
+      <c r="M143" s="71">
+        <v>15.62</v>
+      </c>
+    </row>
+    <row r="144" spans="1:14">
+      <c r="A144" s="59">
+        <v>2</v>
+      </c>
+      <c r="B144" s="59">
+        <v>26</v>
+      </c>
+      <c r="C144" s="59">
+        <v>158</v>
+      </c>
+      <c r="D144" s="59">
+        <v>0</v>
+      </c>
+      <c r="E144" s="59" t="str">
+        <f t="shared" si="3"/>
+        <v>Compra</v>
+      </c>
+      <c r="F144" s="75">
+        <v>365.86865</v>
+      </c>
+      <c r="J144" s="68">
+        <v>41906.903368055559</v>
+      </c>
+      <c r="K144" s="73">
+        <v>12.694599999999999</v>
+      </c>
+      <c r="L144" s="73">
+        <v>12.69455</v>
+      </c>
+      <c r="M144" s="71">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145" spans="1:13">
+      <c r="A145" s="59">
+        <v>2</v>
+      </c>
+      <c r="B145" s="59">
+        <v>26</v>
+      </c>
+      <c r="C145" s="59">
+        <v>159</v>
+      </c>
+      <c r="D145" s="59">
+        <v>0</v>
+      </c>
+      <c r="E145" s="59" t="str">
+        <f t="shared" si="3"/>
+        <v>Compra</v>
+      </c>
+      <c r="F145" s="75">
+        <v>365.86865</v>
+      </c>
+      <c r="J145" s="68">
+        <v>42662.903900462959</v>
+      </c>
+      <c r="K145" s="73">
+        <v>13.118</v>
+      </c>
+      <c r="L145" s="73">
+        <v>13.118</v>
+      </c>
+      <c r="M145" s="71">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Afegida tab Simulació venda.
</commit_message>
<xml_diff>
--- a/Docs/CompresOriginals.xlsx
+++ b/Docs/CompresOriginals.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4507"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="80" yWindow="130" windowWidth="19140" windowHeight="7830"/>
+    <workbookView xWindow="80" yWindow="130" windowWidth="19140" windowHeight="7830" firstSheet="9" activeTab="16"/>
   </bookViews>
   <sheets>
     <sheet name="PigTributa" sheetId="22" r:id="rId1"/>
@@ -23,6 +23,7 @@
     <sheet name="Sheet3" sheetId="5" r:id="rId14"/>
     <sheet name="Sheet2" sheetId="4" r:id="rId15"/>
     <sheet name="Sheet1" sheetId="1" r:id="rId16"/>
+    <sheet name="Proves-20020607" sheetId="23" r:id="rId17"/>
   </sheets>
   <calcPr calcId="125725"/>
 </workbook>
@@ -256,7 +257,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="822" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="836" uniqueCount="213">
   <si>
     <t>Compra</t>
   </si>
@@ -883,6 +884,18 @@
   </si>
   <si>
     <t>Americ-&gt;</t>
+  </si>
+  <si>
+    <t>Part act</t>
+  </si>
+  <si>
+    <t>PU Orig</t>
+  </si>
+  <si>
+    <t>Id C Orig</t>
+  </si>
+  <si>
+    <t>Id Comp</t>
   </si>
 </sst>
 </file>
@@ -9779,6 +9792,350 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="D3:Q22"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="5" width="8.7265625" style="59"/>
+    <col min="6" max="6" width="9.81640625" style="59" customWidth="1"/>
+    <col min="7" max="7" width="12.08984375" style="59" customWidth="1"/>
+    <col min="8" max="8" width="8.7265625" style="59"/>
+    <col min="9" max="9" width="14.7265625" style="59" customWidth="1"/>
+    <col min="10" max="16" width="8.7265625" style="59"/>
+    <col min="17" max="17" width="10.26953125" style="59" bestFit="1" customWidth="1"/>
+    <col min="18" max="16384" width="8.7265625" style="59"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="4:17" ht="18.5" customHeight="1">
+      <c r="E3" s="152">
+        <v>26</v>
+      </c>
+      <c r="F3" s="152" t="s">
+        <v>2</v>
+      </c>
+      <c r="G3" s="266">
+        <v>41439</v>
+      </c>
+      <c r="H3" s="152">
+        <v>249.34710000000001</v>
+      </c>
+      <c r="I3" s="59">
+        <f>+H3</f>
+        <v>249.34710000000001</v>
+      </c>
+    </row>
+    <row r="4" spans="4:17" ht="18.5" customHeight="1">
+      <c r="E4" s="275">
+        <v>28</v>
+      </c>
+      <c r="F4" s="275" t="s">
+        <v>5</v>
+      </c>
+      <c r="G4" s="276">
+        <v>41794</v>
+      </c>
+      <c r="H4" s="275">
+        <v>249</v>
+      </c>
+      <c r="I4" s="61">
+        <f>+I3-H4</f>
+        <v>0.34710000000001173</v>
+      </c>
+    </row>
+    <row r="5" spans="4:17" ht="18.5" customHeight="1">
+      <c r="E5" s="152">
+        <v>31</v>
+      </c>
+      <c r="F5" s="152" t="s">
+        <v>2</v>
+      </c>
+      <c r="G5" s="266">
+        <v>41976</v>
+      </c>
+      <c r="H5" s="152">
+        <v>264.18049999999999</v>
+      </c>
+      <c r="I5" s="59">
+        <f>+I4+H5</f>
+        <v>264.52760000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="4:17" ht="18.5" customHeight="1">
+      <c r="E6" s="275">
+        <v>91</v>
+      </c>
+      <c r="F6" s="275" t="s">
+        <v>5</v>
+      </c>
+      <c r="G6" s="276">
+        <v>42201</v>
+      </c>
+      <c r="H6" s="275">
+        <v>259.52999999999997</v>
+      </c>
+      <c r="I6" s="61">
+        <f>+I5-H6</f>
+        <v>4.997600000000034</v>
+      </c>
+      <c r="K6" s="59">
+        <f>+H4+H6</f>
+        <v>508.53</v>
+      </c>
+    </row>
+    <row r="8" spans="4:17">
+      <c r="D8" s="59">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="4:17">
+      <c r="E9" s="152">
+        <v>7</v>
+      </c>
+      <c r="F9" s="152" t="s">
+        <v>0</v>
+      </c>
+      <c r="G9" s="266">
+        <v>41492</v>
+      </c>
+      <c r="H9" s="152">
+        <v>24.091999999999999</v>
+      </c>
+      <c r="I9" s="59">
+        <f>H9</f>
+        <v>24.091999999999999</v>
+      </c>
+      <c r="J9" s="59">
+        <f>+I9-H11</f>
+        <v>9.0919999999999987</v>
+      </c>
+    </row>
+    <row r="10" spans="4:17">
+      <c r="E10" s="152">
+        <v>39</v>
+      </c>
+      <c r="F10" s="152" t="s">
+        <v>2</v>
+      </c>
+      <c r="G10" s="266">
+        <v>41673</v>
+      </c>
+      <c r="H10" s="152">
+        <v>3.1440000000000001</v>
+      </c>
+      <c r="I10" s="59">
+        <f>I9+H10</f>
+        <v>27.235999999999997</v>
+      </c>
+      <c r="J10" s="59">
+        <f>+J9+H10</f>
+        <v>12.235999999999999</v>
+      </c>
+      <c r="K10" s="59">
+        <f>L10-J9</f>
+        <v>2.9080000000000013</v>
+      </c>
+      <c r="L10" s="59">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="4:17">
+      <c r="E11" s="275">
+        <v>40</v>
+      </c>
+      <c r="F11" s="275" t="s">
+        <v>5</v>
+      </c>
+      <c r="G11" s="276">
+        <v>42047</v>
+      </c>
+      <c r="H11" s="275">
+        <v>15</v>
+      </c>
+      <c r="I11" s="59">
+        <f>I10-H11</f>
+        <v>12.235999999999997</v>
+      </c>
+      <c r="K11" s="59">
+        <f>+L11-J9-H10</f>
+        <v>0.76400000000000112</v>
+      </c>
+      <c r="L11" s="59">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="4:17">
+      <c r="E12" s="152">
+        <v>96</v>
+      </c>
+      <c r="F12" s="152" t="s">
+        <v>2</v>
+      </c>
+      <c r="G12" s="266">
+        <v>42208</v>
+      </c>
+      <c r="H12" s="152">
+        <v>10.042999999999999</v>
+      </c>
+      <c r="I12" s="59">
+        <f t="shared" ref="I12:I13" si="0">I11+H12</f>
+        <v>22.278999999999996</v>
+      </c>
+    </row>
+    <row r="13" spans="4:17">
+      <c r="E13" s="152">
+        <v>104</v>
+      </c>
+      <c r="F13" s="152" t="s">
+        <v>2</v>
+      </c>
+      <c r="G13" s="266">
+        <v>42311</v>
+      </c>
+      <c r="H13" s="152">
+        <v>4.7E-2</v>
+      </c>
+      <c r="I13" s="59">
+        <f t="shared" si="0"/>
+        <v>22.325999999999997</v>
+      </c>
+      <c r="L13" s="59" t="s">
+        <v>212</v>
+      </c>
+      <c r="M13" s="59" t="s">
+        <v>211</v>
+      </c>
+      <c r="N13" s="59" t="s">
+        <v>209</v>
+      </c>
+      <c r="O13" s="59" t="s">
+        <v>175</v>
+      </c>
+      <c r="P13" s="59" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="14" spans="4:17">
+      <c r="L14" s="59">
+        <v>7</v>
+      </c>
+      <c r="M14" s="59">
+        <v>7</v>
+      </c>
+      <c r="N14" s="59">
+        <v>9.0920000000000005</v>
+      </c>
+      <c r="O14" s="59">
+        <v>9.0920000000000005</v>
+      </c>
+      <c r="P14" s="299">
+        <v>250.44120000000001</v>
+      </c>
+      <c r="Q14" s="60">
+        <f>O14*P14</f>
+        <v>2277.0113904000004</v>
+      </c>
+    </row>
+    <row r="15" spans="4:17">
+      <c r="L15" s="59">
+        <v>39</v>
+      </c>
+      <c r="M15" s="59">
+        <v>37</v>
+      </c>
+      <c r="N15" s="59">
+        <f>H10</f>
+        <v>3.1440000000000001</v>
+      </c>
+      <c r="O15" s="59">
+        <v>75</v>
+      </c>
+      <c r="P15" s="299">
+        <v>13.03</v>
+      </c>
+      <c r="Q15" s="60">
+        <f>O15*P15</f>
+        <v>977.25</v>
+      </c>
+    </row>
+    <row r="16" spans="4:17">
+      <c r="L16" s="59">
+        <v>96</v>
+      </c>
+      <c r="M16" s="59">
+        <v>7</v>
+      </c>
+      <c r="N16" s="59">
+        <f>H12</f>
+        <v>10.042999999999999</v>
+      </c>
+      <c r="O16" s="152">
+        <v>12.914</v>
+      </c>
+      <c r="P16" s="299">
+        <f>P14</f>
+        <v>250.44120000000001</v>
+      </c>
+      <c r="Q16" s="60">
+        <f>O16*P16</f>
+        <v>3234.1976568</v>
+      </c>
+    </row>
+    <row r="17" spans="6:17">
+      <c r="L17" s="59">
+        <v>104</v>
+      </c>
+      <c r="M17" s="59">
+        <v>37</v>
+      </c>
+      <c r="N17" s="59">
+        <f>H13</f>
+        <v>4.7E-2</v>
+      </c>
+      <c r="O17" s="152">
+        <v>1.746</v>
+      </c>
+      <c r="P17" s="299">
+        <v>13.03</v>
+      </c>
+      <c r="Q17" s="60">
+        <f>O17*P17</f>
+        <v>22.75038</v>
+      </c>
+    </row>
+    <row r="18" spans="6:17">
+      <c r="G18" s="60">
+        <v>8544.69</v>
+      </c>
+      <c r="Q18" s="60">
+        <f>SUM(Q14:Q17)</f>
+        <v>6511.2094272000004</v>
+      </c>
+    </row>
+    <row r="19" spans="6:17">
+      <c r="G19" s="59">
+        <v>8494.8799999999992</v>
+      </c>
+    </row>
+    <row r="20" spans="6:17">
+      <c r="G20" s="60">
+        <f>+G18-G19</f>
+        <v>49.81000000000131</v>
+      </c>
+    </row>
+    <row r="22" spans="6:17">
+      <c r="F22" s="60">
+        <v>274.68</v>
+      </c>
+      <c r="G22" s="60">
+        <v>6132.72</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:T58"/>

</xml_diff>